<commit_message>
Add Furqan Ahmad; make Collaborate page free of locations and university names; refresh areas sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SYNTERA-member-areas.xlsx
+++ b/SYNTERA-member-areas.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1772,7 +1772,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Muhammad Irfan Aslam</t>
+          <t>Furqan Ahmad</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1782,12 +1782,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>University of Education, Lahore</t>
+          <t>Northwestern Polytechnical University, Xi'an</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Natural Language Processing; Deep Learning; Artificial Intelligence; Image Processing; Machine Learning</t>
+          <t>AIoT; Edge computing; TinyML; SDN &amp; network automation; Smart healthcare</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -1798,8 +1798,16 @@
       <c r="G28" s="3" t="inlineStr"/>
       <c r="H28" s="3" t="inlineStr"/>
       <c r="I28" s="3" t="inlineStr"/>
-      <c r="J28" s="3" t="inlineStr"/>
-      <c r="K28" s="3" t="inlineStr"/>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1812,7 +1820,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Sepehr Amooeinejad</t>
+          <t>Muhammad Irfan Aslam</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1822,12 +1830,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>School of Information Systems, Queensland University of Technology, Brisbane, QLD</t>
+          <t>University of Education, Lahore</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning; Sports Injury Prediction; Bibliometrics; Digital Health; Sports Analytics</t>
+          <t>Natural Language Processing; Deep Learning; Artificial Intelligence; Image Processing; Machine Learning</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -1852,7 +1860,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Ghalib Nadeem</t>
+          <t>Sepehr Amooeinejad</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1862,36 +1870,24 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Department of Computer Science, Huazhong University of Science and Technology, Wuhan</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr"/>
+          <t>School of Information Systems, Queensland University of Technology, Brisbane, QLD</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Machine Learning; Sports Injury Prediction; Bibliometrics; Digital Health; Sports Analytics</t>
+        </is>
+      </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G30" s="3" t="inlineStr"/>
+      <c r="H30" s="3" t="inlineStr"/>
       <c r="I30" s="3" t="inlineStr"/>
-      <c r="J30" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="K30" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="J30" s="3" t="inlineStr"/>
+      <c r="K30" s="3" t="inlineStr"/>
       <c r="L30" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1904,7 +1900,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nida Ali</t>
+          <t>Ghalib Nadeem</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1914,24 +1910,36 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Department of Skill Development and Leadership, The University of Lahore, Lahore</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>Corpus Linguistics; English for Specific Purposes; Text Analysis; Computer-Assisted Language Learning; Applied Linguistics</t>
-        </is>
-      </c>
-      <c r="F31" s="3" t="inlineStr"/>
-      <c r="G31" s="3" t="inlineStr"/>
-      <c r="H31" s="3" t="inlineStr"/>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J31" s="3" t="inlineStr"/>
-      <c r="K31" s="3" t="inlineStr"/>
+          <t>Department of Computer Science, Huazhong University of Science and Technology, Wuhan</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr"/>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr"/>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1944,7 +1952,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Hina Mehboob</t>
+          <t>Nida Ali</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1954,23 +1962,23 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>National University of Sciences and Technology (NUST), Islamabad</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Department of Skill Development and Leadership, The University of Lahore, Lahore</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Corpus Linguistics; English for Specific Purposes; Text Analysis; Computer-Assisted Language Learning; Applied Linguistics</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr"/>
       <c r="G32" s="3" t="inlineStr"/>
       <c r="H32" s="3" t="inlineStr"/>
-      <c r="I32" s="3" t="inlineStr"/>
-      <c r="J32" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr"/>
       <c r="K32" s="3" t="inlineStr"/>
       <c r="L32" s="3" t="inlineStr">
         <is>
@@ -1984,7 +1992,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Hasanga Uyanhewage</t>
+          <t>Hina Mehboob</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1994,15 +2002,15 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Tesco Mobile, Tesco UK</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Software engineering; Human–AI interaction; AI governance; Privacy &amp; data protection; Trust &amp; decision-making</t>
-        </is>
-      </c>
-      <c r="F33" s="3" t="inlineStr"/>
+          <t>National University of Sciences and Technology (NUST), Islamabad</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G33" s="3" t="inlineStr"/>
       <c r="H33" s="3" t="inlineStr"/>
       <c r="I33" s="3" t="inlineStr"/>
@@ -2024,7 +2032,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Malak Emziane</t>
+          <t>Hasanga Uyanhewage</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2034,19 +2042,15 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>University of Tipaza</t>
+          <t>Tesco Mobile, Tesco UK</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Quantum cryptography; IoT; AI; Secure 5G/6G networks</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Software engineering; Human–AI interaction; AI governance; Privacy &amp; data protection; Trust &amp; decision-making</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr"/>
       <c r="G34" s="3" t="inlineStr"/>
       <c r="H34" s="3" t="inlineStr"/>
       <c r="I34" s="3" t="inlineStr"/>
@@ -2055,11 +2059,7 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K34" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K34" s="3" t="inlineStr"/>
       <c r="L34" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -2072,7 +2072,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Mohamadali Rezaeimanesh</t>
+          <t>Malak Emziane</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2082,15 +2082,19 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>School of Information Systems, Queensland University of Technology (QUT), Brisbane, QLD</t>
+          <t>University of Tipaza</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning; Artificial Intelligence; Extended Reality (XR); Cloud Computing</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr"/>
+          <t>Quantum cryptography; IoT; AI; Secure 5G/6G networks</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G35" s="3" t="inlineStr"/>
       <c r="H35" s="3" t="inlineStr"/>
       <c r="I35" s="3" t="inlineStr"/>
@@ -2099,7 +2103,11 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K35" s="3" t="inlineStr"/>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -2112,7 +2120,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Amir H. Malekijoo</t>
+          <t>Mohamadali Rezaeimanesh</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2122,19 +2130,15 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Faculty of Computer Engineering, Department of Computer Engineering, Semnan University</t>
+          <t>School of Information Systems, Queensland University of Technology (QUT), Brisbane, QLD</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Artificial Intelligence; Reinforcement Learning; Human-Computer Interaction; Pattern Recognition; Decision Making Theory</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Machine Learning; Artificial Intelligence; Extended Reality (XR); Cloud Computing</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr"/>
       <c r="G36" s="3" t="inlineStr"/>
       <c r="H36" s="3" t="inlineStr"/>
       <c r="I36" s="3" t="inlineStr"/>
@@ -2156,7 +2160,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Thiwanka Kaushalya Nagasanga</t>
+          <t>Amir H. Malekijoo</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2166,15 +2170,19 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>CQUniversity Australia</t>
+          <t>Faculty of Computer Engineering, Department of Computer Engineering, Semnan University</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Explainable AI (XAI); Human-AI Decision-Making; AI Agents; Software Engineering; Project Management</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr"/>
+          <t>Artificial Intelligence; Reinforcement Learning; Human-Computer Interaction; Pattern Recognition; Decision Making Theory</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G37" s="3" t="inlineStr"/>
       <c r="H37" s="3" t="inlineStr"/>
       <c r="I37" s="3" t="inlineStr"/>
@@ -2196,7 +2204,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Meerab Fatima</t>
+          <t>Thiwanka Kaushalya Nagasanga</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2206,23 +2214,23 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Department of Computer Science, FAST National University of Computer and Emerging Sciences (FAST-NUCES)</t>
+          <t>CQUniversity Australia</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Recommender Systems; Natural Language Processing; Semantic Search and Information Retrieval; Large Language Models; Career and Skill-Gap Analysis</t>
+          <t>Explainable AI (XAI); Human-AI Decision-Making; AI Agents; Software Engineering; Project Management</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr"/>
       <c r="G38" s="3" t="inlineStr"/>
       <c r="H38" s="3" t="inlineStr"/>
-      <c r="I38" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J38" s="3" t="inlineStr"/>
+      <c r="I38" s="3" t="inlineStr"/>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K38" s="3" t="inlineStr"/>
       <c r="L38" s="3" t="inlineStr">
         <is>
@@ -2236,7 +2244,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Malahat Mardani</t>
+          <t>Meerab Fatima</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2246,27 +2254,23 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Babol Noshirvani University of Technology</t>
+          <t>Department of Computer Science, FAST National University of Computer and Emerging Sciences (FAST-NUCES)</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning &amp; Deep Learning; Computer Vision; Medical Image Analysis; Biomedical Signal Processing (EEG); Model Reliability &amp; Generalization</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Recommender Systems; Natural Language Processing; Semantic Search and Information Retrieval; Large Language Models; Career and Skill-Gap Analysis</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr"/>
       <c r="G39" s="3" t="inlineStr"/>
       <c r="H39" s="3" t="inlineStr"/>
-      <c r="I39" s="3" t="inlineStr"/>
-      <c r="J39" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr"/>
       <c r="K39" s="3" t="inlineStr"/>
       <c r="L39" s="3" t="inlineStr">
         <is>
@@ -2280,7 +2284,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Mounes Mardani</t>
+          <t>Malahat Mardani</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2324,7 +2328,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Ramsha Khan</t>
+          <t>Mounes Mardani</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2334,12 +2338,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>University of Lahore</t>
+          <t>Babol Noshirvani University of Technology</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>AI for health; Biomedical research; Molecular medicine; Virology &amp; infectious diseases; AI in healthcare; Bioinformatics</t>
+          <t>Machine Learning &amp; Deep Learning; Computer Vision; Medical Image Analysis; Biomedical Signal Processing (EEG); Model Reliability &amp; Generalization</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
@@ -2350,7 +2354,11 @@
       <c r="G41" s="3" t="inlineStr"/>
       <c r="H41" s="3" t="inlineStr"/>
       <c r="I41" s="3" t="inlineStr"/>
-      <c r="J41" s="3" t="inlineStr"/>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K41" s="3" t="inlineStr"/>
       <c r="L41" s="3" t="inlineStr">
         <is>
@@ -2364,7 +2372,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Ali Hasnain</t>
+          <t>Ramsha Khan</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2374,12 +2382,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Department of Software Engineering, University of Sahiwal</t>
+          <t>University of Lahore</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Computer vision; Medical AI; Large language models; Agentic AI; Deep learning</t>
+          <t>AI for health; Biomedical research; Molecular medicine; Virology &amp; infectious diseases; AI in healthcare; Bioinformatics</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
@@ -2387,18 +2395,10 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G42" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G42" s="3" t="inlineStr"/>
       <c r="H42" s="3" t="inlineStr"/>
       <c r="I42" s="3" t="inlineStr"/>
-      <c r="J42" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="J42" s="3" t="inlineStr"/>
       <c r="K42" s="3" t="inlineStr"/>
       <c r="L42" s="3" t="inlineStr">
         <is>
@@ -2412,7 +2412,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Bilal Aslam</t>
+          <t>Ali Hasnain</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2420,10 +2420,14 @@
           <t>Students &amp; Researchers</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Department of Software Engineering, University of Sahiwal</t>
+        </is>
+      </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Machine learning; Deep learning; Healthcare AI; IoMT; Trustworthy AI</t>
+          <t>Computer vision; Medical AI; Large language models; Agentic AI; Deep learning</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
@@ -2431,7 +2435,11 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr"/>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="H43" s="3" t="inlineStr"/>
       <c r="I43" s="3" t="inlineStr"/>
       <c r="J43" s="3" t="inlineStr">
@@ -2440,7 +2448,11 @@
         </is>
       </c>
       <c r="K43" s="3" t="inlineStr"/>
-      <c r="L43" s="3" t="inlineStr"/>
+      <c r="L43" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2448,7 +2460,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Aittezaz Ahmad</t>
+          <t>Bilal Aslam</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2459,10 +2471,14 @@
       <c r="D44" t="inlineStr"/>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Reliability Engineering; Artificial Intelligence; Risk Assessment; Machine Learning–Assisted Optimization; Intelligent Monitoring</t>
-        </is>
-      </c>
-      <c r="F44" s="3" t="inlineStr"/>
+          <t>Machine learning; Deep learning; Healthcare AI; IoMT; Trustworthy AI</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G44" s="3" t="inlineStr"/>
       <c r="H44" s="3" t="inlineStr"/>
       <c r="I44" s="3" t="inlineStr"/>
@@ -2472,54 +2488,86 @@
         </is>
       </c>
       <c r="K44" s="3" t="inlineStr"/>
-      <c r="L44" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr"/>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="L44" s="3" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Aittezaz Ahmad</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Students &amp; Researchers</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Reliability Engineering; Artificial Intelligence; Risk Assessment; Machine Learning–Assisted Optimization; Intelligent Monitoring</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr"/>
+      <c r="G45" s="3" t="inlineStr"/>
+      <c r="H45" s="3" t="inlineStr"/>
+      <c r="I45" s="3" t="inlineStr"/>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr"/>
+      <c r="L45" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr"/>
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>Total (current)</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr"/>
-      <c r="D46" s="4" t="inlineStr"/>
-      <c r="E46" s="4" t="inlineStr"/>
-      <c r="F46" s="4">
-        <f>COUNTIF(F2:F44,"x")</f>
+      <c r="C47" s="4" t="inlineStr"/>
+      <c r="D47" s="4" t="inlineStr"/>
+      <c r="E47" s="4" t="inlineStr"/>
+      <c r="F47" s="4">
+        <f>COUNTIF(F2:F45,"x")</f>
         <v/>
       </c>
-      <c r="G46" s="4">
-        <f>COUNTIF(G2:G44,"x")</f>
+      <c r="G47" s="4">
+        <f>COUNTIF(G2:G45,"x")</f>
         <v/>
       </c>
-      <c r="H46" s="4">
-        <f>COUNTIF(H2:H44,"x")</f>
+      <c r="H47" s="4">
+        <f>COUNTIF(H2:H45,"x")</f>
         <v/>
       </c>
-      <c r="I46" s="4">
-        <f>COUNTIF(I2:I44,"x")</f>
+      <c r="I47" s="4">
+        <f>COUNTIF(I2:I45,"x")</f>
         <v/>
       </c>
-      <c r="J46" s="4">
-        <f>COUNTIF(J2:J44,"x")</f>
+      <c r="J47" s="4">
+        <f>COUNTIF(J2:J45,"x")</f>
         <v/>
       </c>
-      <c r="K46" s="4">
-        <f>COUNTIF(K2:K44,"x")</f>
+      <c r="K47" s="4">
+        <f>COUNTIF(K2:K45,"x")</f>
         <v/>
       </c>
-      <c r="L46" s="4">
-        <f>COUNTIF(L2:L44,"x")</f>
+      <c r="L47" s="4">
+        <f>COUNTIF(L2:L45,"x")</f>
         <v/>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" t="inlineStr"/>
-      <c r="B47" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr"/>
+      <c r="B48" t="inlineStr">
         <is>
           <t>Mark "x" in each area a member belongs to</t>
         </is>

</xml_diff>

<commit_message>
Wathiq Mansoor: AUIB main affiliation (Iraq), Macquarie secondary; refresh areas sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SYNTERA-member-areas.xlsx
+++ b/SYNTERA-member-areas.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Dr. Tanja Pavleska</t>
+          <t>Professor Wathiq Mansoor</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -762,12 +762,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Laboratory for Open Systems and Networks, Jožef Stefan Institute, Ljubljana</t>
+          <t>College of Engineering, American University in Baghdad (AUIB); Honorary Professor, Macquarie University</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Cybersecurity for AI; AI for cybersecurity; Trustworthy &amp; explainable AI; Critical infrastructure security; Industrial automation &amp; digital twins; Threat intelligence &amp; digital forensics; Digital policies &amp; regulatory frameworks; Computational trust &amp; reputation systems</t>
+          <t>Biomedical signal processing; Image processing; Parallel processing; Smart technologies; Computer engineering</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -782,11 +782,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr"/>
       <c r="I6" s="3" t="inlineStr"/>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="J6" s="3" t="inlineStr"/>
       <c r="K6" s="3" t="inlineStr"/>
       <c r="L6" s="3" t="inlineStr">
         <is>
@@ -800,7 +796,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dr. Shiva Ilkhani Zadeh</t>
+          <t>Dr. Tanja Pavleska</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -810,19 +806,31 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Business School, Business and Law Department, Bournemouth University</t>
+          <t>Laboratory for Open Systems and Networks, Jožef Stefan Institute, Ljubljana</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Leadership; Sustainability; AI in tourism; Nudging</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr"/>
+          <t>Cybersecurity for AI; AI for cybersecurity; Trustworthy &amp; explainable AI; Critical infrastructure security; Industrial automation &amp; digital twins; Threat intelligence &amp; digital forensics; Digital policies &amp; regulatory frameworks; Computational trust &amp; reputation systems</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr"/>
-      <c r="J7" s="3" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K7" s="3" t="inlineStr"/>
       <c r="L7" s="3" t="inlineStr">
         <is>
@@ -836,7 +844,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Dr. Mostafa Kamalpour, PhD</t>
+          <t>Dr. Shiva Ilkhani Zadeh</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -846,28 +854,20 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>School of Information Systems, Faculty of Science, Queensland University of Technology</t>
+          <t>Business School, Business and Law Department, Bournemouth University</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Digital Health; Service Science; Social Media</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Leadership; Sustainability; AI in tourism; Nudging</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr"/>
       <c r="G8" s="3" t="inlineStr"/>
       <c r="H8" s="3" t="inlineStr"/>
       <c r="I8" s="3" t="inlineStr"/>
       <c r="J8" s="3" t="inlineStr"/>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K8" s="3" t="inlineStr"/>
       <c r="L8" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -880,7 +880,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Dr. Hanem Ellethy</t>
+          <t>Dr. Mostafa Kamalpour, PhD</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -890,12 +890,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>School of Electrical Engineering and Computer Science (EECS), The University of Queensland</t>
+          <t>School of Information Systems, Faculty of Science, Queensland University of Technology</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Applied AI &amp; intelligent systems; Trustworthy, explainable &amp; human-centred AI; AI in healthcare &amp; medical imaging; Generative AI in education; AI-enhanced learning; AI reliability, robustness &amp; real-world deployment</t>
+          <t>Digital Health; Service Science; Social Media</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -905,16 +905,8 @@
       </c>
       <c r="G9" s="3" t="inlineStr"/>
       <c r="H9" s="3" t="inlineStr"/>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J9" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I9" s="3" t="inlineStr"/>
+      <c r="J9" s="3" t="inlineStr"/>
       <c r="K9" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -932,7 +924,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dr. Mana Mirzaei</t>
+          <t>Dr. Hanem Ellethy</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -942,12 +934,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>University of the Sunshine Coast, Sunshine Coast, Queensland</t>
+          <t>School of Electrical Engineering and Computer Science (EECS), The University of Queensland</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>AI; Business data analysis; Machine learning; Optimisation</t>
+          <t>Applied AI &amp; intelligent systems; Trustworthy, explainable &amp; human-centred AI; AI in healthcare &amp; medical imaging; Generative AI in education; AI-enhanced learning; AI reliability, robustness &amp; real-world deployment</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -956,11 +948,7 @@
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr"/>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="H10" s="3" t="inlineStr"/>
       <c r="I10" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -971,7 +959,11 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr"/>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -984,7 +976,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dr. Syed Fawad M. Zaidi</t>
+          <t>Dr. Mana Mirzaei</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -994,12 +986,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Torrens University Australia</t>
+          <t>University of the Sunshine Coast, Sunshine Coast, Queensland</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Artificial intelligence &amp; intelligent systems; Human-centred design &amp; design thinking; Serious games &amp; immersive learning technologies; Digital health &amp; health informatics; Learning analytics &amp; educational innovation</t>
+          <t>AI; Business data analysis; Machine learning; Optimisation</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1008,13 +1000,21 @@
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr"/>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K11" s="3" t="inlineStr"/>
       <c r="L11" s="3" t="inlineStr">
         <is>
@@ -1028,22 +1028,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Hassan Ahmed</t>
+          <t>Dr. Syed Fawad M. Zaidi</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Team Lead</t>
+          <t>Scientific Advisory Board</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Department of Computer Science, National University of Computer and Emerging Sciences (FAST-NUCES), Chiniot-Faisalabad Campus</t>
+          <t>Torrens University Australia</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Cybersecurity; Deep Learning; NLP; XAI; LLMs; Computer Vision</t>
+          <t>Artificial intelligence &amp; intelligent systems; Human-centred design &amp; design thinking; Serious games &amp; immersive learning technologies; Digital health &amp; health informatics; Learning analytics &amp; educational innovation</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -1051,32 +1051,20 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" s="3" t="inlineStr"/>
       <c r="I12" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="L12" s="3" t="inlineStr"/>
+      <c r="J12" s="3" t="inlineStr"/>
+      <c r="K12" s="3" t="inlineStr"/>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1084,7 +1072,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sadegh Rajaei</t>
+          <t>Hassan Ahmed</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1094,12 +1082,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Department of Electrical and Computer Engineering, Babol Noshirvani University of Technology, Babol, Iran</t>
+          <t>Department of Computer Science, National University of Computer and Emerging Sciences (FAST-NUCES), Chiniot-Faisalabad Campus</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning; Deep Learning; Data Mining; NLP; Computer Vision</t>
+          <t>Cybersecurity; Deep Learning; NLP; XAI; LLMs; Computer Vision</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -1107,8 +1095,16 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="3" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1119,12 +1115,12 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr"/>
-      <c r="L13" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1132,38 +1128,42 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Hilda Jemutai Bitok</t>
+          <t>Sadegh Rajaei</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Students &amp; Researchers</t>
+          <t>Team Lead</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>School of Science, Technology and Engineering, University of the Sunshine Coast, QLD</t>
+          <t>Department of Electrical and Computer Engineering, Babol Noshirvani University of Technology, Babol, Iran</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>IoV; Vehicular Communication; Machine Learning; Blockchain</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr"/>
+          <t>Machine Learning; Deep Learning; Data Mining; NLP; Computer Vision</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G14" s="3" t="inlineStr"/>
       <c r="H14" s="3" t="inlineStr"/>
-      <c r="I14" s="3" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K14" s="3" t="inlineStr"/>
       <c r="L14" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Abdul Mateen</t>
+          <t>Hilda Jemutai Bitok</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1186,29 +1186,33 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Department of Computer Science, National University of Computer and Emerging Sciences (FAST-NUCES), Chiniot-Faisalabad Campus</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>School of Science, Technology and Engineering, University of the Sunshine Coast, QLD</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>IoV; Vehicular Communication; Machine Learning; Blockchain</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr"/>
       <c r="G15" s="3" t="inlineStr"/>
       <c r="H15" s="3" t="inlineStr"/>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I15" s="3" t="inlineStr"/>
       <c r="J15" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="K15" s="3" t="inlineStr"/>
-      <c r="L15" s="3" t="inlineStr"/>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1216,7 +1220,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abdullah Khan</t>
+          <t>Abdul Mateen</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1226,29 +1230,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Department of Computer Science, University of Wah, Wah Cantt</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Cybersecurity; Deep Learning; NLP; Applications of AI</t>
-        </is>
-      </c>
+          <t>Department of Computer Science, National University of Computer and Emerging Sciences (FAST-NUCES), Chiniot-Faisalabad Campus</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+      <c r="H16" s="3" t="inlineStr"/>
       <c r="I16" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1259,16 +1251,8 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="L16" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K16" s="3" t="inlineStr"/>
+      <c r="L16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1276,7 +1260,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Svetlana Kolos</t>
+          <t>Abdullah Khan</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1286,12 +1270,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Torrens University Australia</t>
+          <t>Department of Computer Science, University of Wah, Wah Cantt</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Artificial Intelligence; Information Systems; Digital Transformation; Health Informatics; Decision Support Systems</t>
+          <t>Cybersecurity; Deep Learning; NLP; Applications of AI</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1304,10 +1288,26 @@
           <t>x</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr"/>
-      <c r="I17" s="3" t="inlineStr"/>
-      <c r="J17" s="3" t="inlineStr"/>
-      <c r="K17" s="3" t="inlineStr"/>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1320,7 +1320,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Samia Mujahid</t>
+          <t>Svetlana Kolos</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1330,12 +1330,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Department of Computer Science, National University of Computer and Emerging Sciences (FAST-NUCES), Chiniot-Faisalabad Campus</t>
+          <t>Torrens University Australia</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>NLP; Healthcare; LLMs; Ethics and Privacy; AI</t>
+          <t>Artificial Intelligence; Information Systems; Digital Transformation; Health Informatics; Decision Support Systems</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -1343,18 +1343,14 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr"/>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr"/>
       <c r="I18" s="3" t="inlineStr"/>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="J18" s="3" t="inlineStr"/>
       <c r="K18" s="3" t="inlineStr"/>
       <c r="L18" s="3" t="inlineStr">
         <is>
@@ -1368,7 +1364,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Jie Zhu</t>
+          <t>Samia Mujahid</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1378,17 +1374,25 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>The University of Queensland</t>
+          <t>Department of Computer Science, National University of Computer and Emerging Sciences (FAST-NUCES), Chiniot-Faisalabad Campus</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Information Systems; Artificial Intelligence; Digital Transformation; Business Analytics; Human–AI Collaboration</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr"/>
+          <t>NLP; Healthcare; LLMs; Ethics and Privacy; AI</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G19" s="3" t="inlineStr"/>
-      <c r="H19" s="3" t="inlineStr"/>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I19" s="3" t="inlineStr"/>
       <c r="J19" s="3" t="inlineStr">
         <is>
@@ -1408,7 +1412,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Bisma Ali</t>
+          <t>Saviz Zarei</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1418,12 +1422,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>School of Electrical Engineering and Computer Science (SEECS), NUST Islamabad</t>
+          <t>University of the Sunshine Coast, Sunshine Coast, Queensland; Queensland Health</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Deep Learning; Computational Intelligence; Computer Vision &amp; Multimodal Learning</t>
+          <t>Health informatics; Decision support systems; Predictive modelling; Simulation modelling; Digital twins for healthcare</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1431,13 +1435,13 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr"/>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="H20" s="3" t="inlineStr"/>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I20" s="3" t="inlineStr"/>
       <c r="J20" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1456,7 +1460,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Manar Makki Shaalan</t>
+          <t>Jie Zhu</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1466,12 +1470,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>University of Babylon, Babylon</t>
+          <t>The University of Queensland</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Graph theory; Domination theory; Network reliability</t>
+          <t>Information Systems; Artificial Intelligence; Digital Transformation; Business Analytics; Human–AI Collaboration</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr"/>
@@ -1496,7 +1500,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Javeria Iqbal</t>
+          <t>Bisma Ali</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1506,10 +1510,14 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Department of Computer Science, National University of Computer and Emerging Sciences, Islamabad</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr"/>
+          <t>School of Electrical Engineering and Computer Science (SEECS), NUST Islamabad</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Deep Learning; Computational Intelligence; Computer Vision &amp; Multimodal Learning</t>
+        </is>
+      </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1540,7 +1548,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Damilare Ogunjobi</t>
+          <t>Manar Makki Shaalan</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1550,21 +1558,17 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Department of Data Science and Analytics, BI Norwegian Business School, Oslo</t>
+          <t>University of Babylon, Babylon</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Cybersecurity; Machine Learning; Networking &amp; IoT; Artificial Intelligence; Trustworthy AI</t>
+          <t>Graph theory; Domination theory; Network reliability</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr"/>
       <c r="G23" s="3" t="inlineStr"/>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="H23" s="3" t="inlineStr"/>
       <c r="I23" s="3" t="inlineStr"/>
       <c r="J23" s="3" t="inlineStr">
         <is>
@@ -1584,7 +1588,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Nazmul Hossain</t>
+          <t>Javeria Iqbal</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1594,28 +1598,28 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Penston Academy of International Studies, Dhaka</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Cybersecurity; Network Security; Data Privacy and Security; Wireless Networks and Communication Protocols; Human-AI Interactions</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr"/>
+          <t>Department of Computer Science, National University of Computer and Emerging Sciences, Islamabad</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G24" s="3" t="inlineStr"/>
       <c r="H24" s="3" t="inlineStr"/>
-      <c r="I24" s="3" t="inlineStr"/>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K24" s="3" t="inlineStr"/>
       <c r="L24" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1628,7 +1632,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Arooj Fatima</t>
+          <t>Damilare Ogunjobi</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1638,36 +1642,28 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Department of Computer Science, University of Wah, Wah Cantt; Govt. Graduate College for Women, Chakwal</t>
+          <t>Department of Data Science and Analytics, BI Norwegian Business School, Oslo</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning; Deep Learning; Cybersecurity; Explainable AI (XAI); Trustworthy AI</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Cybersecurity; Machine Learning; Networking &amp; IoT; Artificial Intelligence; Trustworthy AI</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr"/>
       <c r="G25" s="3" t="inlineStr"/>
-      <c r="H25" s="3" t="inlineStr"/>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr"/>
       <c r="J25" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="K25" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K25" s="3" t="inlineStr"/>
       <c r="L25" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1680,7 +1676,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Tobias Romano</t>
+          <t>Nazmul Hossain</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1690,32 +1686,28 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>UNICEN</t>
+          <t>Penston Academy of International Studies, Dhaka</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Agriculture; Computer Vision; Machine Learning; Robotics; Autonomous Systems</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Cybersecurity; Network Security; Data Privacy and Security; Wireless Networks and Communication Protocols; Human-AI Interactions</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr"/>
       <c r="G26" s="3" t="inlineStr"/>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="H26" s="3" t="inlineStr"/>
       <c r="I26" s="3" t="inlineStr"/>
       <c r="J26" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="K26" s="3" t="inlineStr"/>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1728,7 +1720,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Shiva Jahanaray</t>
+          <t>Arooj Fatima</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1738,12 +1730,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Tafakor Pishro Asredade Parsian, Babol</t>
+          <t>Department of Computer Science, University of Wah, Wah Cantt; Govt. Graduate College for Women, Chakwal</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Artificial Intelligence; Machine Learning; Deep Learning; Multimodal Learning; Biomedical AI</t>
+          <t>Machine Learning; Deep Learning; Cybersecurity; Explainable AI (XAI); Trustworthy AI</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -1753,13 +1745,21 @@
       </c>
       <c r="G27" s="3" t="inlineStr"/>
       <c r="H27" s="3" t="inlineStr"/>
-      <c r="I27" s="3" t="inlineStr"/>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="K27" s="3" t="inlineStr"/>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L27" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1772,7 +1772,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Furqan Ahmad</t>
+          <t>Tobias Romano</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1782,12 +1782,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Northwestern Polytechnical University, Xi'an</t>
+          <t>UNICEN</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>AIoT; Edge computing; TinyML; SDN &amp; network automation; Smart healthcare</t>
+          <t>Agriculture; Computer Vision; Machine Learning; Robotics; Autonomous Systems</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -1796,18 +1796,18 @@
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr"/>
-      <c r="H28" s="3" t="inlineStr"/>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I28" s="3" t="inlineStr"/>
       <c r="J28" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="K28" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K28" s="3" t="inlineStr"/>
       <c r="L28" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1820,7 +1820,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Muhammad Irfan Aslam</t>
+          <t>Shiva Jahanaray</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1830,12 +1830,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>University of Education, Lahore</t>
+          <t>Tafakor Pishro Asredade Parsian, Babol</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Natural Language Processing; Deep Learning; Artificial Intelligence; Image Processing; Machine Learning</t>
+          <t>Artificial Intelligence; Machine Learning; Deep Learning; Multimodal Learning; Biomedical AI</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -1846,7 +1846,11 @@
       <c r="G29" s="3" t="inlineStr"/>
       <c r="H29" s="3" t="inlineStr"/>
       <c r="I29" s="3" t="inlineStr"/>
-      <c r="J29" s="3" t="inlineStr"/>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K29" s="3" t="inlineStr"/>
       <c r="L29" s="3" t="inlineStr">
         <is>
@@ -1860,7 +1864,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Sepehr Amooeinejad</t>
+          <t>Furqan Ahmad</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1870,12 +1874,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>School of Information Systems, Queensland University of Technology, Brisbane, QLD</t>
+          <t>Northwestern Polytechnical University, Xi'an</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning; Sports Injury Prediction; Bibliometrics; Digital Health; Sports Analytics</t>
+          <t>AIoT; Edge computing; TinyML; SDN &amp; network automation; Smart healthcare</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -1886,8 +1890,16 @@
       <c r="G30" s="3" t="inlineStr"/>
       <c r="H30" s="3" t="inlineStr"/>
       <c r="I30" s="3" t="inlineStr"/>
-      <c r="J30" s="3" t="inlineStr"/>
-      <c r="K30" s="3" t="inlineStr"/>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1900,7 +1912,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Ghalib Nadeem</t>
+          <t>Muhammad Irfan Aslam</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1910,36 +1922,24 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Department of Computer Science, Huazhong University of Science and Technology, Wuhan</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr"/>
+          <t>University of Education, Lahore</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Natural Language Processing; Deep Learning; Artificial Intelligence; Image Processing; Machine Learning</t>
+        </is>
+      </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G31" s="3" t="inlineStr"/>
+      <c r="H31" s="3" t="inlineStr"/>
       <c r="I31" s="3" t="inlineStr"/>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="K31" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="J31" s="3" t="inlineStr"/>
+      <c r="K31" s="3" t="inlineStr"/>
       <c r="L31" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1952,7 +1952,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Nida Ali</t>
+          <t>Sepehr Amooeinejad</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1962,22 +1962,22 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Department of Skill Development and Leadership, The University of Lahore, Lahore</t>
+          <t>School of Information Systems, Queensland University of Technology, Brisbane, QLD</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Corpus Linguistics; English for Specific Purposes; Text Analysis; Computer-Assisted Language Learning; Applied Linguistics</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="inlineStr"/>
+          <t>Machine Learning; Sports Injury Prediction; Bibliometrics; Digital Health; Sports Analytics</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G32" s="3" t="inlineStr"/>
       <c r="H32" s="3" t="inlineStr"/>
-      <c r="I32" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I32" s="3" t="inlineStr"/>
       <c r="J32" s="3" t="inlineStr"/>
       <c r="K32" s="3" t="inlineStr"/>
       <c r="L32" s="3" t="inlineStr">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Hina Mehboob</t>
+          <t>Ghalib Nadeem</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2002,7 +2002,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>National University of Sciences and Technology (NUST), Islamabad</t>
+          <t>Department of Computer Science, Huazhong University of Science and Technology, Wuhan</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr"/>
@@ -2011,15 +2011,27 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr"/>
-      <c r="H33" s="3" t="inlineStr"/>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I33" s="3" t="inlineStr"/>
       <c r="J33" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="K33" s="3" t="inlineStr"/>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -2032,7 +2044,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Hasanga Uyanhewage</t>
+          <t>Nida Ali</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2042,23 +2054,23 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Tesco Mobile, Tesco UK</t>
+          <t>Department of Skill Development and Leadership, The University of Lahore, Lahore</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Software engineering; Human–AI interaction; AI governance; Privacy &amp; data protection; Trust &amp; decision-making</t>
+          <t>Corpus Linguistics; English for Specific Purposes; Text Analysis; Computer-Assisted Language Learning; Applied Linguistics</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr"/>
       <c r="G34" s="3" t="inlineStr"/>
       <c r="H34" s="3" t="inlineStr"/>
-      <c r="I34" s="3" t="inlineStr"/>
-      <c r="J34" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr"/>
       <c r="K34" s="3" t="inlineStr"/>
       <c r="L34" s="3" t="inlineStr">
         <is>
@@ -2072,7 +2084,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Malak Emziane</t>
+          <t>Hina Mehboob</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2082,14 +2094,10 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>University of Tipaza</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>Quantum cryptography; IoT; AI; Secure 5G/6G networks</t>
-        </is>
-      </c>
+          <t>National University of Sciences and Technology (NUST), Islamabad</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -2103,11 +2111,7 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K35" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K35" s="3" t="inlineStr"/>
       <c r="L35" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -2120,7 +2124,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Mohamadali Rezaeimanesh</t>
+          <t>Hasanga Uyanhewage</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2130,12 +2134,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>School of Information Systems, Queensland University of Technology (QUT), Brisbane, QLD</t>
+          <t>Tesco Mobile, Tesco UK</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning; Artificial Intelligence; Extended Reality (XR); Cloud Computing</t>
+          <t>Software engineering; Human–AI interaction; AI governance; Privacy &amp; data protection; Trust &amp; decision-making</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr"/>
@@ -2160,7 +2164,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Amir H. Malekijoo</t>
+          <t>Malak Emziane</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2170,12 +2174,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Faculty of Computer Engineering, Department of Computer Engineering, Semnan University</t>
+          <t>University of Tipaza</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Artificial Intelligence; Reinforcement Learning; Human-Computer Interaction; Pattern Recognition; Decision Making Theory</t>
+          <t>Quantum cryptography; IoT; AI; Secure 5G/6G networks</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
@@ -2191,7 +2195,11 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K37" s="3" t="inlineStr"/>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -2204,7 +2212,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Thiwanka Kaushalya Nagasanga</t>
+          <t>Mohamadali Rezaeimanesh</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2214,12 +2222,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>CQUniversity Australia</t>
+          <t>School of Information Systems, Queensland University of Technology (QUT), Brisbane, QLD</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Explainable AI (XAI); Human-AI Decision-Making; AI Agents; Software Engineering; Project Management</t>
+          <t>Machine Learning; Artificial Intelligence; Extended Reality (XR); Cloud Computing</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr"/>
@@ -2244,7 +2252,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Meerab Fatima</t>
+          <t>Amir H. Malekijoo</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2254,23 +2262,27 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Department of Computer Science, FAST National University of Computer and Emerging Sciences (FAST-NUCES)</t>
+          <t>Faculty of Computer Engineering, Department of Computer Engineering, Semnan University</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Recommender Systems; Natural Language Processing; Semantic Search and Information Retrieval; Large Language Models; Career and Skill-Gap Analysis</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr"/>
+          <t>Artificial Intelligence; Reinforcement Learning; Human-Computer Interaction; Pattern Recognition; Decision Making Theory</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G39" s="3" t="inlineStr"/>
       <c r="H39" s="3" t="inlineStr"/>
-      <c r="I39" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J39" s="3" t="inlineStr"/>
+      <c r="I39" s="3" t="inlineStr"/>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K39" s="3" t="inlineStr"/>
       <c r="L39" s="3" t="inlineStr">
         <is>
@@ -2284,7 +2296,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Malahat Mardani</t>
+          <t>Thiwanka Kaushalya Nagasanga</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2294,19 +2306,15 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Babol Noshirvani University of Technology</t>
+          <t>CQUniversity Australia</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning &amp; Deep Learning; Computer Vision; Medical Image Analysis; Biomedical Signal Processing (EEG); Model Reliability &amp; Generalization</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Explainable AI (XAI); Human-AI Decision-Making; AI Agents; Software Engineering; Project Management</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr"/>
       <c r="G40" s="3" t="inlineStr"/>
       <c r="H40" s="3" t="inlineStr"/>
       <c r="I40" s="3" t="inlineStr"/>
@@ -2328,7 +2336,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Mounes Mardani</t>
+          <t>Meerab Fatima</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2338,27 +2346,23 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Babol Noshirvani University of Technology</t>
+          <t>Department of Computer Science, FAST National University of Computer and Emerging Sciences (FAST-NUCES)</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning &amp; Deep Learning; Computer Vision; Medical Image Analysis; Biomedical Signal Processing (EEG); Model Reliability &amp; Generalization</t>
-        </is>
-      </c>
-      <c r="F41" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Recommender Systems; Natural Language Processing; Semantic Search and Information Retrieval; Large Language Models; Career and Skill-Gap Analysis</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr"/>
       <c r="G41" s="3" t="inlineStr"/>
       <c r="H41" s="3" t="inlineStr"/>
-      <c r="I41" s="3" t="inlineStr"/>
-      <c r="J41" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr"/>
       <c r="K41" s="3" t="inlineStr"/>
       <c r="L41" s="3" t="inlineStr">
         <is>
@@ -2372,7 +2376,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Ramsha Khan</t>
+          <t>Malahat Mardani</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2382,12 +2386,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>University of Lahore</t>
+          <t>Babol Noshirvani University of Technology</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>AI for health; Biomedical research; Molecular medicine; Virology &amp; infectious diseases; AI in healthcare; Bioinformatics</t>
+          <t>Machine Learning &amp; Deep Learning; Computer Vision; Medical Image Analysis; Biomedical Signal Processing (EEG); Model Reliability &amp; Generalization</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
@@ -2398,7 +2402,11 @@
       <c r="G42" s="3" t="inlineStr"/>
       <c r="H42" s="3" t="inlineStr"/>
       <c r="I42" s="3" t="inlineStr"/>
-      <c r="J42" s="3" t="inlineStr"/>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K42" s="3" t="inlineStr"/>
       <c r="L42" s="3" t="inlineStr">
         <is>
@@ -2412,7 +2420,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Ali Hasnain</t>
+          <t>Mounes Mardani</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2422,12 +2430,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Department of Software Engineering, University of Sahiwal</t>
+          <t>Babol Noshirvani University of Technology</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Computer vision; Medical AI; Large language models; Agentic AI; Deep learning</t>
+          <t>Machine Learning &amp; Deep Learning; Computer Vision; Medical Image Analysis; Biomedical Signal Processing (EEG); Model Reliability &amp; Generalization</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
@@ -2435,11 +2443,7 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G43" s="3" t="inlineStr"/>
       <c r="H43" s="3" t="inlineStr"/>
       <c r="I43" s="3" t="inlineStr"/>
       <c r="J43" s="3" t="inlineStr">
@@ -2460,7 +2464,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Bilal Aslam</t>
+          <t>Ramsha Khan</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2468,10 +2472,14 @@
           <t>Students &amp; Researchers</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>University of Lahore</t>
+        </is>
+      </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Machine learning; Deep learning; Healthcare AI; IoMT; Trustworthy AI</t>
+          <t>AI for health; Biomedical research; Molecular medicine; Virology &amp; infectious diseases; AI in healthcare; Bioinformatics</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -2482,13 +2490,13 @@
       <c r="G44" s="3" t="inlineStr"/>
       <c r="H44" s="3" t="inlineStr"/>
       <c r="I44" s="3" t="inlineStr"/>
-      <c r="J44" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="J44" s="3" t="inlineStr"/>
       <c r="K44" s="3" t="inlineStr"/>
-      <c r="L44" s="3" t="inlineStr"/>
+      <c r="L44" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2496,7 +2504,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Aittezaz Ahmad</t>
+          <t>Ali Hasnain</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2504,14 +2512,26 @@
           <t>Students &amp; Researchers</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Department of Software Engineering, University of Sahiwal</t>
+        </is>
+      </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Reliability Engineering; Artificial Intelligence; Risk Assessment; Machine Learning–Assisted Optimization; Intelligent Monitoring</t>
-        </is>
-      </c>
-      <c r="F45" s="3" t="inlineStr"/>
-      <c r="G45" s="3" t="inlineStr"/>
+          <t>Computer vision; Medical AI; Large language models; Agentic AI; Deep learning</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="H45" s="3" t="inlineStr"/>
       <c r="I45" s="3" t="inlineStr"/>
       <c r="J45" s="3" t="inlineStr">
@@ -2526,48 +2546,120 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Bilal Aslam</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Students &amp; Researchers</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>Machine learning; Deep learning; Healthcare AI; IoMT; Trustworthy AI</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr"/>
+      <c r="H46" s="3" t="inlineStr"/>
+      <c r="I46" s="3" t="inlineStr"/>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr"/>
+      <c r="L46" s="3" t="inlineStr"/>
+    </row>
     <row r="47">
-      <c r="A47" s="4" t="inlineStr"/>
-      <c r="B47" s="4" t="inlineStr">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Aittezaz Ahmad</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Students &amp; Researchers</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Reliability Engineering; Artificial Intelligence; Risk Assessment; Machine Learning–Assisted Optimization; Intelligent Monitoring</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr"/>
+      <c r="G47" s="3" t="inlineStr"/>
+      <c r="H47" s="3" t="inlineStr"/>
+      <c r="I47" s="3" t="inlineStr"/>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K47" s="3" t="inlineStr"/>
+      <c r="L47" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr"/>
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>Total (current)</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr"/>
-      <c r="D47" s="4" t="inlineStr"/>
-      <c r="E47" s="4" t="inlineStr"/>
-      <c r="F47" s="4">
-        <f>COUNTIF(F2:F45,"x")</f>
+      <c r="C49" s="4" t="inlineStr"/>
+      <c r="D49" s="4" t="inlineStr"/>
+      <c r="E49" s="4" t="inlineStr"/>
+      <c r="F49" s="4">
+        <f>COUNTIF(F2:F47,"x")</f>
         <v/>
       </c>
-      <c r="G47" s="4">
-        <f>COUNTIF(G2:G45,"x")</f>
+      <c r="G49" s="4">
+        <f>COUNTIF(G2:G47,"x")</f>
         <v/>
       </c>
-      <c r="H47" s="4">
-        <f>COUNTIF(H2:H45,"x")</f>
+      <c r="H49" s="4">
+        <f>COUNTIF(H2:H47,"x")</f>
         <v/>
       </c>
-      <c r="I47" s="4">
-        <f>COUNTIF(I2:I45,"x")</f>
+      <c r="I49" s="4">
+        <f>COUNTIF(I2:I47,"x")</f>
         <v/>
       </c>
-      <c r="J47" s="4">
-        <f>COUNTIF(J2:J45,"x")</f>
+      <c r="J49" s="4">
+        <f>COUNTIF(J2:J47,"x")</f>
         <v/>
       </c>
-      <c r="K47" s="4">
-        <f>COUNTIF(K2:K45,"x")</f>
+      <c r="K49" s="4">
+        <f>COUNTIF(K2:K47,"x")</f>
         <v/>
       </c>
-      <c r="L47" s="4">
-        <f>COUNTIF(L2:L45,"x")</f>
+      <c r="L49" s="4">
+        <f>COUNTIF(L2:L47,"x")</f>
         <v/>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" t="inlineStr"/>
-      <c r="B48" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr">
         <is>
           <t>Mark "x" in each area a member belongs to</t>
         </is>

</xml_diff>

<commit_message>
Iran-based members: Independent Researcher, no flag
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SYNTERA-member-areas.xlsx
+++ b/SYNTERA-member-areas.xlsx
@@ -1138,7 +1138,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Department of Electrical and Computer Engineering, Babol Noshirvani University of Technology, Babol, Iran</t>
+          <t>Independent Researcher</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Tafakor Pishro Asredade Parsian, Babol</t>
+          <t>Independent Researcher</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2262,7 +2262,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Faculty of Computer Engineering, Department of Computer Engineering, Semnan University</t>
+          <t>Independent Researcher</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Babol Noshirvani University of Technology</t>
+          <t>Independent Researcher</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2430,7 +2430,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Babol Noshirvani University of Technology</t>
+          <t>Independent Researcher</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Iraq-based members: remove flag and affiliation
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SYNTERA-member-areas.xlsx
+++ b/SYNTERA-member-areas.xlsx
@@ -762,7 +762,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>College of Engineering, American University in Baghdad (AUIB); Honorary Professor, Macquarie University</t>
+          <t>Macquarie University</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>University of Babylon, Babylon</t>
+          <t>Independent Researcher</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">

</xml_diff>

<commit_message>
China-based members: Independent Researcher, no flag
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SYNTERA-member-areas.xlsx
+++ b/SYNTERA-member-areas.xlsx
@@ -1874,7 +1874,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Northwestern Polytechnical University, Xi'an</t>
+          <t>Independent Researcher</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -2002,7 +2002,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Department of Computer Science, Huazhong University of Science and Technology, Wuhan</t>
+          <t>Independent Researcher</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Add Bisma Nawaz to Students & Researchers
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SYNTERA-member-areas.xlsx
+++ b/SYNTERA-member-areas.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Manar Makki Shaalan</t>
+          <t>Bisma Nawaz</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1558,16 +1558,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Independent Researcher</t>
+          <t>Department of Computer Science, National University of Computer and Emerging Sciences, Pakistan</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Graph theory; Domination theory; Network reliability</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr"/>
-      <c r="G23" s="3" t="inlineStr"/>
+          <t>Natural language processing; Deep learning; Medical imaging; Computer vision</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="H23" s="3" t="inlineStr"/>
       <c r="I23" s="3" t="inlineStr"/>
       <c r="J23" s="3" t="inlineStr">
@@ -1588,7 +1596,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Javeria Iqbal</t>
+          <t>Manar Makki Shaalan</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1598,22 +1606,18 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Department of Computer Science, National University of Computer and Emerging Sciences, Islamabad</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Independent Researcher</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Graph theory; Domination theory; Network reliability</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr"/>
       <c r="G24" s="3" t="inlineStr"/>
       <c r="H24" s="3" t="inlineStr"/>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I24" s="3" t="inlineStr"/>
       <c r="J24" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1632,7 +1636,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Damilare Ogunjobi</t>
+          <t>Javeria Iqbal</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1642,22 +1646,22 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Department of Data Science and Analytics, BI Norwegian Business School, Oslo</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Cybersecurity; Machine Learning; Networking &amp; IoT; Artificial Intelligence; Trustworthy AI</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr"/>
+          <t>Department of Computer Science, National University of Computer and Emerging Sciences, Islamabad</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G25" s="3" t="inlineStr"/>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="I25" s="3" t="inlineStr"/>
+      <c r="H25" s="3" t="inlineStr"/>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1676,7 +1680,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Nazmul Hossain</t>
+          <t>Damilare Ogunjobi</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1686,28 +1690,28 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Penston Academy of International Studies, Dhaka</t>
+          <t>Department of Data Science and Analytics, BI Norwegian Business School, Oslo</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Cybersecurity; Network Security; Data Privacy and Security; Wireless Networks and Communication Protocols; Human-AI Interactions</t>
+          <t>Cybersecurity; Machine Learning; Networking &amp; IoT; Artificial Intelligence; Trustworthy AI</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr"/>
       <c r="G26" s="3" t="inlineStr"/>
-      <c r="H26" s="3" t="inlineStr"/>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I26" s="3" t="inlineStr"/>
       <c r="J26" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="K26" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K26" s="3" t="inlineStr"/>
       <c r="L26" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1720,7 +1724,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Arooj Fatima</t>
+          <t>Nazmul Hossain</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1730,26 +1734,18 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Department of Computer Science, University of Wah, Wah Cantt; Govt. Graduate College for Women, Chakwal</t>
+          <t>Penston Academy of International Studies, Dhaka</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning; Deep Learning; Cybersecurity; Explainable AI (XAI); Trustworthy AI</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Cybersecurity; Network Security; Data Privacy and Security; Wireless Networks and Communication Protocols; Human-AI Interactions</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr"/>
       <c r="G27" s="3" t="inlineStr"/>
       <c r="H27" s="3" t="inlineStr"/>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I27" s="3" t="inlineStr"/>
       <c r="J27" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1772,7 +1768,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Tobias Romano</t>
+          <t>Arooj Fatima</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1782,12 +1778,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>UNICEN</t>
+          <t>Department of Computer Science, University of Wah, Wah Cantt; Govt. Graduate College for Women, Chakwal</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Agriculture; Computer Vision; Machine Learning; Robotics; Autonomous Systems</t>
+          <t>Machine Learning; Deep Learning; Cybersecurity; Explainable AI (XAI); Trustworthy AI</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -1796,18 +1792,22 @@
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr"/>
-      <c r="H28" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="I28" s="3" t="inlineStr"/>
+      <c r="H28" s="3" t="inlineStr"/>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="K28" s="3" t="inlineStr"/>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1820,7 +1820,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Shiva Jahanaray</t>
+          <t>Tobias Romano</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1830,12 +1830,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Independent Researcher</t>
+          <t>UNICEN</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Artificial Intelligence; Machine Learning; Deep Learning; Multimodal Learning; Biomedical AI</t>
+          <t>Agriculture; Computer Vision; Machine Learning; Robotics; Autonomous Systems</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -1844,7 +1844,11 @@
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr"/>
-      <c r="H29" s="3" t="inlineStr"/>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I29" s="3" t="inlineStr"/>
       <c r="J29" s="3" t="inlineStr">
         <is>
@@ -1864,7 +1868,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Furqan Ahmad</t>
+          <t>Shiva Jahanaray</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1879,7 +1883,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>AIoT; Edge computing; TinyML; SDN &amp; network automation; Smart healthcare</t>
+          <t>Artificial Intelligence; Machine Learning; Deep Learning; Multimodal Learning; Biomedical AI</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -1895,11 +1899,7 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K30" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K30" s="3" t="inlineStr"/>
       <c r="L30" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Muhammad Irfan Aslam</t>
+          <t>Furqan Ahmad</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1922,12 +1922,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>University of Education, Lahore</t>
+          <t>Independent Researcher</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Natural Language Processing; Deep Learning; Artificial Intelligence; Image Processing; Machine Learning</t>
+          <t>AIoT; Edge computing; TinyML; SDN &amp; network automation; Smart healthcare</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -1938,8 +1938,16 @@
       <c r="G31" s="3" t="inlineStr"/>
       <c r="H31" s="3" t="inlineStr"/>
       <c r="I31" s="3" t="inlineStr"/>
-      <c r="J31" s="3" t="inlineStr"/>
-      <c r="K31" s="3" t="inlineStr"/>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1952,7 +1960,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Sepehr Amooeinejad</t>
+          <t>Muhammad Irfan Aslam</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1962,12 +1970,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>School of Information Systems, Queensland University of Technology, Brisbane, QLD</t>
+          <t>University of Education, Lahore</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning; Sports Injury Prediction; Bibliometrics; Digital Health; Sports Analytics</t>
+          <t>Natural Language Processing; Deep Learning; Artificial Intelligence; Image Processing; Machine Learning</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -1992,7 +2000,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Ghalib Nadeem</t>
+          <t>Sepehr Amooeinejad</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2002,36 +2010,24 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Independent Researcher</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr"/>
+          <t>School of Information Systems, Queensland University of Technology, Brisbane, QLD</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Machine Learning; Sports Injury Prediction; Bibliometrics; Digital Health; Sports Analytics</t>
+        </is>
+      </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G33" s="3" t="inlineStr"/>
+      <c r="H33" s="3" t="inlineStr"/>
       <c r="I33" s="3" t="inlineStr"/>
-      <c r="J33" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="K33" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="J33" s="3" t="inlineStr"/>
+      <c r="K33" s="3" t="inlineStr"/>
       <c r="L33" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -2044,7 +2040,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Nida Ali</t>
+          <t>Ghalib Nadeem</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2054,24 +2050,36 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Department of Skill Development and Leadership, The University of Lahore, Lahore</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>Corpus Linguistics; English for Specific Purposes; Text Analysis; Computer-Assisted Language Learning; Applied Linguistics</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr"/>
-      <c r="G34" s="3" t="inlineStr"/>
-      <c r="H34" s="3" t="inlineStr"/>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J34" s="3" t="inlineStr"/>
-      <c r="K34" s="3" t="inlineStr"/>
+          <t>Independent Researcher</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr"/>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -2084,7 +2092,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Hina Mehboob</t>
+          <t>Nida Ali</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2094,23 +2102,23 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>National University of Sciences and Technology (NUST), Islamabad</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr"/>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Department of Skill Development and Leadership, The University of Lahore, Lahore</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Corpus Linguistics; English for Specific Purposes; Text Analysis; Computer-Assisted Language Learning; Applied Linguistics</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr"/>
       <c r="G35" s="3" t="inlineStr"/>
       <c r="H35" s="3" t="inlineStr"/>
-      <c r="I35" s="3" t="inlineStr"/>
-      <c r="J35" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr"/>
       <c r="K35" s="3" t="inlineStr"/>
       <c r="L35" s="3" t="inlineStr">
         <is>
@@ -2124,7 +2132,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Hasanga Uyanhewage</t>
+          <t>Hina Mehboob</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2134,15 +2142,15 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Tesco Mobile, Tesco UK</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>Software engineering; Human–AI interaction; AI governance; Privacy &amp; data protection; Trust &amp; decision-making</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr"/>
+          <t>National University of Sciences and Technology (NUST), Islamabad</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G36" s="3" t="inlineStr"/>
       <c r="H36" s="3" t="inlineStr"/>
       <c r="I36" s="3" t="inlineStr"/>
@@ -2164,7 +2172,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Malak Emziane</t>
+          <t>Hasanga Uyanhewage</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2174,19 +2182,15 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>University of Tipaza</t>
+          <t>Tesco Mobile, Tesco UK</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Quantum cryptography; IoT; AI; Secure 5G/6G networks</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Software engineering; Human–AI interaction; AI governance; Privacy &amp; data protection; Trust &amp; decision-making</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr"/>
       <c r="G37" s="3" t="inlineStr"/>
       <c r="H37" s="3" t="inlineStr"/>
       <c r="I37" s="3" t="inlineStr"/>
@@ -2195,11 +2199,7 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K37" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K37" s="3" t="inlineStr"/>
       <c r="L37" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Mohamadali Rezaeimanesh</t>
+          <t>Malak Emziane</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2222,15 +2222,19 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>School of Information Systems, Queensland University of Technology (QUT), Brisbane, QLD</t>
+          <t>University of Tipaza</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning; Artificial Intelligence; Extended Reality (XR); Cloud Computing</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr"/>
+          <t>Quantum cryptography; IoT; AI; Secure 5G/6G networks</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G38" s="3" t="inlineStr"/>
       <c r="H38" s="3" t="inlineStr"/>
       <c r="I38" s="3" t="inlineStr"/>
@@ -2239,7 +2243,11 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K38" s="3" t="inlineStr"/>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L38" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -2252,7 +2260,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Amir H. Malekijoo</t>
+          <t>Mohamadali Rezaeimanesh</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2262,19 +2270,15 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Independent Researcher</t>
+          <t>School of Information Systems, Queensland University of Technology (QUT), Brisbane, QLD</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Artificial Intelligence; Reinforcement Learning; Human-Computer Interaction; Pattern Recognition; Decision Making Theory</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Machine Learning; Artificial Intelligence; Extended Reality (XR); Cloud Computing</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr"/>
       <c r="G39" s="3" t="inlineStr"/>
       <c r="H39" s="3" t="inlineStr"/>
       <c r="I39" s="3" t="inlineStr"/>
@@ -2296,7 +2300,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Thiwanka Kaushalya Nagasanga</t>
+          <t>Amir H. Malekijoo</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2306,15 +2310,19 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>CQUniversity Australia</t>
+          <t>Independent Researcher</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Explainable AI (XAI); Human-AI Decision-Making; AI Agents; Software Engineering; Project Management</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="inlineStr"/>
+          <t>Artificial Intelligence; Reinforcement Learning; Human-Computer Interaction; Pattern Recognition; Decision Making Theory</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G40" s="3" t="inlineStr"/>
       <c r="H40" s="3" t="inlineStr"/>
       <c r="I40" s="3" t="inlineStr"/>
@@ -2336,7 +2344,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Meerab Fatima</t>
+          <t>Thiwanka Kaushalya Nagasanga</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2346,23 +2354,23 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Department of Computer Science, FAST National University of Computer and Emerging Sciences (FAST-NUCES)</t>
+          <t>CQUniversity Australia</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Recommender Systems; Natural Language Processing; Semantic Search and Information Retrieval; Large Language Models; Career and Skill-Gap Analysis</t>
+          <t>Explainable AI (XAI); Human-AI Decision-Making; AI Agents; Software Engineering; Project Management</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr"/>
       <c r="G41" s="3" t="inlineStr"/>
       <c r="H41" s="3" t="inlineStr"/>
-      <c r="I41" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J41" s="3" t="inlineStr"/>
+      <c r="I41" s="3" t="inlineStr"/>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K41" s="3" t="inlineStr"/>
       <c r="L41" s="3" t="inlineStr">
         <is>
@@ -2376,7 +2384,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Malahat Mardani</t>
+          <t>Meerab Fatima</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2386,27 +2394,23 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Independent Researcher</t>
+          <t>Department of Computer Science, FAST National University of Computer and Emerging Sciences (FAST-NUCES)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning &amp; Deep Learning; Computer Vision; Medical Image Analysis; Biomedical Signal Processing (EEG); Model Reliability &amp; Generalization</t>
-        </is>
-      </c>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Recommender Systems; Natural Language Processing; Semantic Search and Information Retrieval; Large Language Models; Career and Skill-Gap Analysis</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr"/>
       <c r="G42" s="3" t="inlineStr"/>
       <c r="H42" s="3" t="inlineStr"/>
-      <c r="I42" s="3" t="inlineStr"/>
-      <c r="J42" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr"/>
       <c r="K42" s="3" t="inlineStr"/>
       <c r="L42" s="3" t="inlineStr">
         <is>
@@ -2420,7 +2424,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Mounes Mardani</t>
+          <t>Malahat Mardani</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2464,7 +2468,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Ramsha Khan</t>
+          <t>Mounes Mardani</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2474,12 +2478,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>University of Lahore</t>
+          <t>Independent Researcher</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>AI for health; Biomedical research; Molecular medicine; Virology &amp; infectious diseases; AI in healthcare; Bioinformatics</t>
+          <t>Machine Learning &amp; Deep Learning; Computer Vision; Medical Image Analysis; Biomedical Signal Processing (EEG); Model Reliability &amp; Generalization</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -2490,7 +2494,11 @@
       <c r="G44" s="3" t="inlineStr"/>
       <c r="H44" s="3" t="inlineStr"/>
       <c r="I44" s="3" t="inlineStr"/>
-      <c r="J44" s="3" t="inlineStr"/>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K44" s="3" t="inlineStr"/>
       <c r="L44" s="3" t="inlineStr">
         <is>
@@ -2504,7 +2512,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Ali Hasnain</t>
+          <t>Ramsha Khan</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2514,12 +2522,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Department of Software Engineering, University of Sahiwal</t>
+          <t>University of Lahore</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Computer vision; Medical AI; Large language models; Agentic AI; Deep learning</t>
+          <t>AI for health; Biomedical research; Molecular medicine; Virology &amp; infectious diseases; AI in healthcare; Bioinformatics</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
@@ -2527,18 +2535,10 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G45" s="3" t="inlineStr"/>
       <c r="H45" s="3" t="inlineStr"/>
       <c r="I45" s="3" t="inlineStr"/>
-      <c r="J45" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="J45" s="3" t="inlineStr"/>
       <c r="K45" s="3" t="inlineStr"/>
       <c r="L45" s="3" t="inlineStr">
         <is>
@@ -2552,7 +2552,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Bilal Aslam</t>
+          <t>Ali Hasnain</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2560,10 +2560,14 @@
           <t>Students &amp; Researchers</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Department of Software Engineering, University of Sahiwal</t>
+        </is>
+      </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Machine learning; Deep learning; Healthcare AI; IoMT; Trustworthy AI</t>
+          <t>Computer vision; Medical AI; Large language models; Agentic AI; Deep learning</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
@@ -2571,7 +2575,11 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G46" s="3" t="inlineStr"/>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="H46" s="3" t="inlineStr"/>
       <c r="I46" s="3" t="inlineStr"/>
       <c r="J46" s="3" t="inlineStr">
@@ -2580,7 +2588,11 @@
         </is>
       </c>
       <c r="K46" s="3" t="inlineStr"/>
-      <c r="L46" s="3" t="inlineStr"/>
+      <c r="L46" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2588,7 +2600,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Aittezaz Ahmad</t>
+          <t>Bilal Aslam</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2599,10 +2611,14 @@
       <c r="D47" t="inlineStr"/>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Reliability Engineering; Artificial Intelligence; Risk Assessment; Machine Learning–Assisted Optimization; Intelligent Monitoring</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="inlineStr"/>
+          <t>Machine learning; Deep learning; Healthcare AI; IoMT; Trustworthy AI</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G47" s="3" t="inlineStr"/>
       <c r="H47" s="3" t="inlineStr"/>
       <c r="I47" s="3" t="inlineStr"/>
@@ -2612,54 +2628,86 @@
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr"/>
-      <c r="L47" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr"/>
-      <c r="B49" s="4" t="inlineStr">
+      <c r="L47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Aittezaz Ahmad</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Students &amp; Researchers</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Reliability Engineering; Artificial Intelligence; Risk Assessment; Machine Learning–Assisted Optimization; Intelligent Monitoring</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr"/>
+      <c r="G48" s="3" t="inlineStr"/>
+      <c r="H48" s="3" t="inlineStr"/>
+      <c r="I48" s="3" t="inlineStr"/>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K48" s="3" t="inlineStr"/>
+      <c r="L48" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr"/>
+      <c r="B50" s="4" t="inlineStr">
         <is>
           <t>Total (current)</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr"/>
-      <c r="D49" s="4" t="inlineStr"/>
-      <c r="E49" s="4" t="inlineStr"/>
-      <c r="F49" s="4">
-        <f>COUNTIF(F2:F47,"x")</f>
+      <c r="C50" s="4" t="inlineStr"/>
+      <c r="D50" s="4" t="inlineStr"/>
+      <c r="E50" s="4" t="inlineStr"/>
+      <c r="F50" s="4">
+        <f>COUNTIF(F2:F48,"x")</f>
         <v/>
       </c>
-      <c r="G49" s="4">
-        <f>COUNTIF(G2:G47,"x")</f>
+      <c r="G50" s="4">
+        <f>COUNTIF(G2:G48,"x")</f>
         <v/>
       </c>
-      <c r="H49" s="4">
-        <f>COUNTIF(H2:H47,"x")</f>
+      <c r="H50" s="4">
+        <f>COUNTIF(H2:H48,"x")</f>
         <v/>
       </c>
-      <c r="I49" s="4">
-        <f>COUNTIF(I2:I47,"x")</f>
+      <c r="I50" s="4">
+        <f>COUNTIF(I2:I48,"x")</f>
         <v/>
       </c>
-      <c r="J49" s="4">
-        <f>COUNTIF(J2:J47,"x")</f>
+      <c r="J50" s="4">
+        <f>COUNTIF(J2:J48,"x")</f>
         <v/>
       </c>
-      <c r="K49" s="4">
-        <f>COUNTIF(K2:K47,"x")</f>
+      <c r="K50" s="4">
+        <f>COUNTIF(K2:K48,"x")</f>
         <v/>
       </c>
-      <c r="L49" s="4">
-        <f>COUNTIF(L2:L47,"x")</f>
+      <c r="L50" s="4">
+        <f>COUNTIF(L2:L48,"x")</f>
         <v/>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-      <c r="B50" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr">
         <is>
           <t>Mark "x" in each area a member belongs to</t>
         </is>

</xml_diff>

<commit_message>
Remove Wathiq Mansoor from the site
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SYNTERA-member-areas.xlsx
+++ b/SYNTERA-member-areas.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Member areas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Member areas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -752,7 +752,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Professor Wathiq Mansoor</t>
+          <t>Dr. Tanja Pavleska</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -762,12 +762,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Macquarie University</t>
+          <t>Laboratory for Open Systems and Networks, Jožef Stefan Institute, Ljubljana</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Biomedical signal processing; Image processing; Parallel processing; Smart technologies; Computer engineering</t>
+          <t>Cybersecurity for AI; AI for cybersecurity; Trustworthy &amp; explainable AI; Critical infrastructure security; Industrial automation &amp; digital twins; Threat intelligence &amp; digital forensics; Digital policies &amp; regulatory frameworks; Computational trust &amp; reputation systems</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -782,7 +782,11 @@
       </c>
       <c r="H6" s="3" t="inlineStr"/>
       <c r="I6" s="3" t="inlineStr"/>
-      <c r="J6" s="3" t="inlineStr"/>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K6" s="3" t="inlineStr"/>
       <c r="L6" s="3" t="inlineStr">
         <is>
@@ -796,7 +800,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dr. Tanja Pavleska</t>
+          <t>Dr. Shiva Ilkhani Zadeh</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -806,31 +810,19 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Laboratory for Open Systems and Networks, Jožef Stefan Institute, Ljubljana</t>
+          <t>Business School, Business and Law Department, Bournemouth University</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Cybersecurity for AI; AI for cybersecurity; Trustworthy &amp; explainable AI; Critical infrastructure security; Industrial automation &amp; digital twins; Threat intelligence &amp; digital forensics; Digital policies &amp; regulatory frameworks; Computational trust &amp; reputation systems</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="G7" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Leadership; Sustainability; AI in tourism; Nudging</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr"/>
+      <c r="G7" s="3" t="inlineStr"/>
       <c r="H7" s="3" t="inlineStr"/>
       <c r="I7" s="3" t="inlineStr"/>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="J7" s="3" t="inlineStr"/>
       <c r="K7" s="3" t="inlineStr"/>
       <c r="L7" s="3" t="inlineStr">
         <is>
@@ -844,7 +836,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Dr. Shiva Ilkhani Zadeh</t>
+          <t>Dr. Mostafa Kamalpour, PhD</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -854,20 +846,28 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Business School, Business and Law Department, Bournemouth University</t>
+          <t>School of Information Systems, Faculty of Science, Queensland University of Technology</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Leadership; Sustainability; AI in tourism; Nudging</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr"/>
+          <t>Digital Health; Service Science; Social Media</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G8" s="3" t="inlineStr"/>
       <c r="H8" s="3" t="inlineStr"/>
       <c r="I8" s="3" t="inlineStr"/>
       <c r="J8" s="3" t="inlineStr"/>
-      <c r="K8" s="3" t="inlineStr"/>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -880,7 +880,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Dr. Mostafa Kamalpour, PhD</t>
+          <t>Dr. Hanem Ellethy</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -890,12 +890,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>School of Information Systems, Faculty of Science, Queensland University of Technology</t>
+          <t>School of Electrical Engineering and Computer Science (EECS), The University of Queensland</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Digital Health; Service Science; Social Media</t>
+          <t>Applied AI &amp; intelligent systems; Trustworthy, explainable &amp; human-centred AI; AI in healthcare &amp; medical imaging; Generative AI in education; AI-enhanced learning; AI reliability, robustness &amp; real-world deployment</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -905,8 +905,16 @@
       </c>
       <c r="G9" s="3" t="inlineStr"/>
       <c r="H9" s="3" t="inlineStr"/>
-      <c r="I9" s="3" t="inlineStr"/>
-      <c r="J9" s="3" t="inlineStr"/>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -924,7 +932,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dr. Hanem Ellethy</t>
+          <t>Dr. Mana Mirzaei</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -934,12 +942,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>School of Electrical Engineering and Computer Science (EECS), The University of Queensland</t>
+          <t>University of the Sunshine Coast, Sunshine Coast, Queensland</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Applied AI &amp; intelligent systems; Trustworthy, explainable &amp; human-centred AI; AI in healthcare &amp; medical imaging; Generative AI in education; AI-enhanced learning; AI reliability, robustness &amp; real-world deployment</t>
+          <t>AI; Business data analysis; Machine learning; Optimisation</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -948,7 +956,11 @@
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr"/>
-      <c r="H10" s="3" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -959,11 +971,7 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K10" s="3" t="inlineStr"/>
       <c r="L10" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -976,7 +984,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Dr. Mana Mirzaei</t>
+          <t>Dr. Syed Fawad M. Zaidi</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -986,12 +994,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>University of the Sunshine Coast, Sunshine Coast, Queensland</t>
+          <t>Torrens University Australia</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>AI; Business data analysis; Machine learning; Optimisation</t>
+          <t>Artificial intelligence &amp; intelligent systems; Human-centred design &amp; design thinking; Serious games &amp; immersive learning technologies; Digital health &amp; health informatics; Learning analytics &amp; educational innovation</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1000,21 +1008,13 @@
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="H11" s="3" t="inlineStr"/>
       <c r="I11" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="J11" s="3" t="inlineStr"/>
       <c r="K11" s="3" t="inlineStr"/>
       <c r="L11" s="3" t="inlineStr">
         <is>
@@ -1028,22 +1028,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Dr. Syed Fawad M. Zaidi</t>
+          <t>Hassan Ahmed</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Scientific Advisory Board</t>
+          <t>Team Lead</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Torrens University Australia</t>
+          <t>Department of Computer Science, National University of Computer and Emerging Sciences (FAST-NUCES), Chiniot-Faisalabad Campus</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Artificial intelligence &amp; intelligent systems; Human-centred design &amp; design thinking; Serious games &amp; immersive learning technologies; Digital health &amp; health informatics; Learning analytics &amp; educational innovation</t>
+          <t>Cybersecurity; Deep Learning; NLP; XAI; LLMs; Computer Vision</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -1051,20 +1051,32 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr"/>
-      <c r="H12" s="3" t="inlineStr"/>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr"/>
-      <c r="K12" s="3" t="inlineStr"/>
-      <c r="L12" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1072,7 +1084,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Hassan Ahmed</t>
+          <t>Sadegh Rajaei</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1082,12 +1094,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Department of Computer Science, National University of Computer and Emerging Sciences (FAST-NUCES), Chiniot-Faisalabad Campus</t>
+          <t>Independent Researcher</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Cybersecurity; Deep Learning; NLP; XAI; LLMs; Computer Vision</t>
+          <t>Machine Learning; Deep Learning; Data Mining; NLP; Computer Vision</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -1095,16 +1107,8 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G13" s="3" t="inlineStr"/>
+      <c r="H13" s="3" t="inlineStr"/>
       <c r="I13" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1115,12 +1119,12 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="L13" s="3" t="inlineStr"/>
+      <c r="K13" s="3" t="inlineStr"/>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1128,42 +1132,38 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Sadegh Rajaei</t>
+          <t>Hilda Jemutai Bitok</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Team Lead</t>
+          <t>Students &amp; Researchers</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Independent Researcher</t>
+          <t>School of Science, Technology and Engineering, University of the Sunshine Coast, QLD</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning; Deep Learning; Data Mining; NLP; Computer Vision</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>IoV; Vehicular Communication; Machine Learning; Blockchain</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr"/>
       <c r="G14" s="3" t="inlineStr"/>
       <c r="H14" s="3" t="inlineStr"/>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I14" s="3" t="inlineStr"/>
       <c r="J14" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr"/>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Hilda Jemutai Bitok</t>
+          <t>Abdul Mateen</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1186,33 +1186,29 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>School of Science, Technology and Engineering, University of the Sunshine Coast, QLD</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>IoV; Vehicular Communication; Machine Learning; Blockchain</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr"/>
+          <t>Department of Computer Science, National University of Computer and Emerging Sciences (FAST-NUCES), Chiniot-Faisalabad Campus</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G15" s="3" t="inlineStr"/>
       <c r="H15" s="3" t="inlineStr"/>
-      <c r="I15" s="3" t="inlineStr"/>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="K15" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="L15" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K15" s="3" t="inlineStr"/>
+      <c r="L15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1220,7 +1216,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Abdul Mateen</t>
+          <t>Abdullah Khan</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1230,17 +1226,29 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Department of Computer Science, National University of Computer and Emerging Sciences (FAST-NUCES), Chiniot-Faisalabad Campus</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
+          <t>Department of Computer Science, University of Wah, Wah Cantt</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Cybersecurity; Deep Learning; NLP; Applications of AI</t>
+        </is>
+      </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr"/>
-      <c r="H16" s="3" t="inlineStr"/>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1251,8 +1259,16 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr"/>
-      <c r="L16" s="3" t="inlineStr"/>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1260,7 +1276,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Abdullah Khan</t>
+          <t>Svetlana Kolos</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1270,12 +1286,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Department of Computer Science, University of Wah, Wah Cantt</t>
+          <t>Torrens University Australia</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Cybersecurity; Deep Learning; NLP; Applications of AI</t>
+          <t>Artificial Intelligence; Information Systems; Digital Transformation; Health Informatics; Decision Support Systems</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1288,26 +1304,10 @@
           <t>x</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J17" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="K17" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="H17" s="3" t="inlineStr"/>
+      <c r="I17" s="3" t="inlineStr"/>
+      <c r="J17" s="3" t="inlineStr"/>
+      <c r="K17" s="3" t="inlineStr"/>
       <c r="L17" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1320,7 +1320,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Svetlana Kolos</t>
+          <t>Samia Mujahid</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1330,12 +1330,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Torrens University Australia</t>
+          <t>Department of Computer Science, National University of Computer and Emerging Sciences (FAST-NUCES), Chiniot-Faisalabad Campus</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Artificial Intelligence; Information Systems; Digital Transformation; Health Informatics; Decision Support Systems</t>
+          <t>NLP; Healthcare; LLMs; Ethics and Privacy; AI</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -1343,14 +1343,18 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr"/>
+      <c r="G18" s="3" t="inlineStr"/>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I18" s="3" t="inlineStr"/>
-      <c r="J18" s="3" t="inlineStr"/>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K18" s="3" t="inlineStr"/>
       <c r="L18" s="3" t="inlineStr">
         <is>
@@ -1364,7 +1368,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Samia Mujahid</t>
+          <t>Saviz Zarei</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1374,12 +1378,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Department of Computer Science, National University of Computer and Emerging Sciences (FAST-NUCES), Chiniot-Faisalabad Campus</t>
+          <t>University of the Sunshine Coast, Sunshine Coast, Queensland; Queensland Health</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>NLP; Healthcare; LLMs; Ethics and Privacy; AI</t>
+          <t>Health informatics; Decision support systems; Predictive modelling; Simulation modelling; Digital twins for healthcare</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1387,12 +1391,12 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr"/>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr"/>
       <c r="I19" s="3" t="inlineStr"/>
       <c r="J19" s="3" t="inlineStr">
         <is>
@@ -1412,7 +1416,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Saviz Zarei</t>
+          <t>Jie Zhu</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1422,24 +1426,16 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>University of the Sunshine Coast, Sunshine Coast, Queensland; Queensland Health</t>
+          <t>The University of Queensland</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Health informatics; Decision support systems; Predictive modelling; Simulation modelling; Digital twins for healthcare</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Information Systems; Artificial Intelligence; Digital Transformation; Business Analytics; Human–AI Collaboration</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr"/>
+      <c r="G20" s="3" t="inlineStr"/>
       <c r="H20" s="3" t="inlineStr"/>
       <c r="I20" s="3" t="inlineStr"/>
       <c r="J20" s="3" t="inlineStr">
@@ -1460,7 +1456,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Jie Zhu</t>
+          <t>Bisma Ali</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1470,18 +1466,26 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>The University of Queensland</t>
+          <t>School of Electrical Engineering and Computer Science (SEECS), NUST Islamabad</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Information Systems; Artificial Intelligence; Digital Transformation; Business Analytics; Human–AI Collaboration</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr"/>
+          <t>Deep Learning; Computational Intelligence; Computer Vision &amp; Multimodal Learning</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G21" s="3" t="inlineStr"/>
       <c r="H21" s="3" t="inlineStr"/>
-      <c r="I21" s="3" t="inlineStr"/>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1500,7 +1504,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Bisma Ali</t>
+          <t>Bisma Nawaz</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1510,12 +1514,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>School of Electrical Engineering and Computer Science (SEECS), NUST Islamabad</t>
+          <t>Department of Computer Science, National University of Computer and Emerging Sciences, Pakistan</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Deep Learning; Computational Intelligence; Computer Vision &amp; Multimodal Learning</t>
+          <t>Natural language processing; Deep learning; Medical imaging; Computer vision</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -1523,13 +1527,13 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr"/>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="H22" s="3" t="inlineStr"/>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I22" s="3" t="inlineStr"/>
       <c r="J22" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1548,7 +1552,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Bisma Nawaz</t>
+          <t>Manar Makki Shaalan</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1558,24 +1562,16 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Department of Computer Science, National University of Computer and Emerging Sciences, Pakistan</t>
+          <t>Independent Researcher</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Natural language processing; Deep learning; Medical imaging; Computer vision</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Graph theory; Domination theory; Network reliability</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr"/>
+      <c r="G23" s="3" t="inlineStr"/>
       <c r="H23" s="3" t="inlineStr"/>
       <c r="I23" s="3" t="inlineStr"/>
       <c r="J23" s="3" t="inlineStr">
@@ -1596,7 +1592,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Manar Makki Shaalan</t>
+          <t>Javeria Iqbal</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1606,18 +1602,22 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Independent Researcher</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Graph theory; Domination theory; Network reliability</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr"/>
+          <t>Department of Computer Science, National University of Computer and Emerging Sciences, Islamabad</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G24" s="3" t="inlineStr"/>
       <c r="H24" s="3" t="inlineStr"/>
-      <c r="I24" s="3" t="inlineStr"/>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1636,7 +1636,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Javeria Iqbal</t>
+          <t>Damilare Ogunjobi</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1646,22 +1646,22 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Department of Computer Science, National University of Computer and Emerging Sciences, Islamabad</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Department of Data Science and Analytics, BI Norwegian Business School, Oslo</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Cybersecurity; Machine Learning; Networking &amp; IoT; Artificial Intelligence; Trustworthy AI</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr"/>
       <c r="G25" s="3" t="inlineStr"/>
-      <c r="H25" s="3" t="inlineStr"/>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr"/>
       <c r="J25" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1680,7 +1680,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Damilare Ogunjobi</t>
+          <t>Nazmul Hossain</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1690,28 +1690,28 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Department of Data Science and Analytics, BI Norwegian Business School, Oslo</t>
+          <t>Penston Academy of International Studies, Dhaka</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Cybersecurity; Machine Learning; Networking &amp; IoT; Artificial Intelligence; Trustworthy AI</t>
+          <t>Cybersecurity; Network Security; Data Privacy and Security; Wireless Networks and Communication Protocols; Human-AI Interactions</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr"/>
       <c r="G26" s="3" t="inlineStr"/>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="H26" s="3" t="inlineStr"/>
       <c r="I26" s="3" t="inlineStr"/>
       <c r="J26" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="K26" s="3" t="inlineStr"/>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Nazmul Hossain</t>
+          <t>Arooj Fatima</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1734,18 +1734,26 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Penston Academy of International Studies, Dhaka</t>
+          <t>Department of Computer Science, University of Wah, Wah Cantt; Govt. Graduate College for Women, Chakwal</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Cybersecurity; Network Security; Data Privacy and Security; Wireless Networks and Communication Protocols; Human-AI Interactions</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr"/>
+          <t>Machine Learning; Deep Learning; Cybersecurity; Explainable AI (XAI); Trustworthy AI</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G27" s="3" t="inlineStr"/>
       <c r="H27" s="3" t="inlineStr"/>
-      <c r="I27" s="3" t="inlineStr"/>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1768,7 +1776,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Arooj Fatima</t>
+          <t>Tobias Romano</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1778,12 +1786,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Department of Computer Science, University of Wah, Wah Cantt; Govt. Graduate College for Women, Chakwal</t>
+          <t>UNICEN</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning; Deep Learning; Cybersecurity; Explainable AI (XAI); Trustworthy AI</t>
+          <t>Agriculture; Computer Vision; Machine Learning; Robotics; Autonomous Systems</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -1792,22 +1800,18 @@
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr"/>
-      <c r="H28" s="3" t="inlineStr"/>
-      <c r="I28" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr"/>
       <c r="J28" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="K28" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K28" s="3" t="inlineStr"/>
       <c r="L28" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1820,7 +1824,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Tobias Romano</t>
+          <t>Shiva Jahanaray</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1830,12 +1834,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>UNICEN</t>
+          <t>Independent Researcher</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Agriculture; Computer Vision; Machine Learning; Robotics; Autonomous Systems</t>
+          <t>Artificial Intelligence; Machine Learning; Deep Learning; Multimodal Learning; Biomedical AI</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -1844,11 +1848,7 @@
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr"/>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="H29" s="3" t="inlineStr"/>
       <c r="I29" s="3" t="inlineStr"/>
       <c r="J29" s="3" t="inlineStr">
         <is>
@@ -1868,7 +1868,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Shiva Jahanaray</t>
+          <t>Furqan Ahmad</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Artificial Intelligence; Machine Learning; Deep Learning; Multimodal Learning; Biomedical AI</t>
+          <t>AIoT; Edge computing; TinyML; SDN &amp; network automation; Smart healthcare</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -1899,7 +1899,11 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K30" s="3" t="inlineStr"/>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1912,7 +1916,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Furqan Ahmad</t>
+          <t>Muhammad Irfan Aslam</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1922,12 +1926,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Independent Researcher</t>
+          <t>University of Education, Lahore</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>AIoT; Edge computing; TinyML; SDN &amp; network automation; Smart healthcare</t>
+          <t>Natural Language Processing; Deep Learning; Artificial Intelligence; Image Processing; Machine Learning</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -1938,16 +1942,8 @@
       <c r="G31" s="3" t="inlineStr"/>
       <c r="H31" s="3" t="inlineStr"/>
       <c r="I31" s="3" t="inlineStr"/>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="K31" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="J31" s="3" t="inlineStr"/>
+      <c r="K31" s="3" t="inlineStr"/>
       <c r="L31" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1960,7 +1956,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Muhammad Irfan Aslam</t>
+          <t>Sepehr Amooeinejad</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1970,12 +1966,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>University of Education, Lahore</t>
+          <t>School of Information Systems, Queensland University of Technology, Brisbane, QLD</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Natural Language Processing; Deep Learning; Artificial Intelligence; Image Processing; Machine Learning</t>
+          <t>Machine Learning; Sports Injury Prediction; Bibliometrics; Digital Health; Sports Analytics</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -2000,7 +1996,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Sepehr Amooeinejad</t>
+          <t>Ghalib Nadeem</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2010,24 +2006,36 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>School of Information Systems, Queensland University of Technology, Brisbane, QLD</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>Machine Learning; Sports Injury Prediction; Bibliometrics; Digital Health; Sports Analytics</t>
-        </is>
-      </c>
+          <t>Independent Researcher</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr"/>
       <c r="F33" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr"/>
-      <c r="H33" s="3" t="inlineStr"/>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I33" s="3" t="inlineStr"/>
-      <c r="J33" s="3" t="inlineStr"/>
-      <c r="K33" s="3" t="inlineStr"/>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -2040,7 +2048,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Ghalib Nadeem</t>
+          <t>Nida Ali</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2050,36 +2058,24 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Independent Researcher</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="I34" s="3" t="inlineStr"/>
-      <c r="J34" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="K34" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Department of Skill Development and Leadership, The University of Lahore, Lahore</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Corpus Linguistics; English for Specific Purposes; Text Analysis; Computer-Assisted Language Learning; Applied Linguistics</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr"/>
+      <c r="G34" s="3" t="inlineStr"/>
+      <c r="H34" s="3" t="inlineStr"/>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr"/>
+      <c r="K34" s="3" t="inlineStr"/>
       <c r="L34" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -2092,7 +2088,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Nida Ali</t>
+          <t>Hina Mehboob</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2102,23 +2098,23 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Department of Skill Development and Leadership, The University of Lahore, Lahore</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>Corpus Linguistics; English for Specific Purposes; Text Analysis; Computer-Assisted Language Learning; Applied Linguistics</t>
-        </is>
-      </c>
-      <c r="F35" s="3" t="inlineStr"/>
+          <t>National University of Sciences and Technology (NUST), Islamabad</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G35" s="3" t="inlineStr"/>
       <c r="H35" s="3" t="inlineStr"/>
-      <c r="I35" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J35" s="3" t="inlineStr"/>
+      <c r="I35" s="3" t="inlineStr"/>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K35" s="3" t="inlineStr"/>
       <c r="L35" s="3" t="inlineStr">
         <is>
@@ -2132,7 +2128,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Hina Mehboob</t>
+          <t>Hasanga Uyanhewage</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2142,15 +2138,15 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>National University of Sciences and Technology (NUST), Islamabad</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Tesco Mobile, Tesco UK</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Software engineering; Human–AI interaction; AI governance; Privacy &amp; data protection; Trust &amp; decision-making</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr"/>
       <c r="G36" s="3" t="inlineStr"/>
       <c r="H36" s="3" t="inlineStr"/>
       <c r="I36" s="3" t="inlineStr"/>
@@ -2172,7 +2168,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Hasanga Uyanhewage</t>
+          <t>Malak Emziane</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2182,15 +2178,19 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Tesco Mobile, Tesco UK</t>
+          <t>University of Tipaza</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Software engineering; Human–AI interaction; AI governance; Privacy &amp; data protection; Trust &amp; decision-making</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr"/>
+          <t>Quantum cryptography; IoT; AI; Secure 5G/6G networks</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G37" s="3" t="inlineStr"/>
       <c r="H37" s="3" t="inlineStr"/>
       <c r="I37" s="3" t="inlineStr"/>
@@ -2199,7 +2199,11 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K37" s="3" t="inlineStr"/>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -2212,7 +2216,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Malak Emziane</t>
+          <t>Mohamadali Rezaeimanesh</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2222,19 +2226,15 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>University of Tipaza</t>
+          <t>School of Information Systems, Queensland University of Technology (QUT), Brisbane, QLD</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Quantum cryptography; IoT; AI; Secure 5G/6G networks</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Machine Learning; Artificial Intelligence; Extended Reality (XR); Cloud Computing</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr"/>
       <c r="G38" s="3" t="inlineStr"/>
       <c r="H38" s="3" t="inlineStr"/>
       <c r="I38" s="3" t="inlineStr"/>
@@ -2243,11 +2243,7 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K38" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K38" s="3" t="inlineStr"/>
       <c r="L38" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -2260,7 +2256,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Mohamadali Rezaeimanesh</t>
+          <t>Amir H. Malekijoo</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2270,15 +2266,19 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>School of Information Systems, Queensland University of Technology (QUT), Brisbane, QLD</t>
+          <t>Independent Researcher</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning; Artificial Intelligence; Extended Reality (XR); Cloud Computing</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr"/>
+          <t>Artificial Intelligence; Reinforcement Learning; Human-Computer Interaction; Pattern Recognition; Decision Making Theory</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G39" s="3" t="inlineStr"/>
       <c r="H39" s="3" t="inlineStr"/>
       <c r="I39" s="3" t="inlineStr"/>
@@ -2300,7 +2300,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Amir H. Malekijoo</t>
+          <t>Thiwanka Kaushalya Nagasanga</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2310,19 +2310,15 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Independent Researcher</t>
+          <t>CQUniversity Australia</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Artificial Intelligence; Reinforcement Learning; Human-Computer Interaction; Pattern Recognition; Decision Making Theory</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Explainable AI (XAI); Human-AI Decision-Making; AI Agents; Software Engineering; Project Management</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr"/>
       <c r="G40" s="3" t="inlineStr"/>
       <c r="H40" s="3" t="inlineStr"/>
       <c r="I40" s="3" t="inlineStr"/>
@@ -2344,7 +2340,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Thiwanka Kaushalya Nagasanga</t>
+          <t>Meerab Fatima</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2354,23 +2350,23 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>CQUniversity Australia</t>
+          <t>Department of Computer Science, FAST National University of Computer and Emerging Sciences (FAST-NUCES)</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Explainable AI (XAI); Human-AI Decision-Making; AI Agents; Software Engineering; Project Management</t>
+          <t>Recommender Systems; Natural Language Processing; Semantic Search and Information Retrieval; Large Language Models; Career and Skill-Gap Analysis</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr"/>
       <c r="G41" s="3" t="inlineStr"/>
       <c r="H41" s="3" t="inlineStr"/>
-      <c r="I41" s="3" t="inlineStr"/>
-      <c r="J41" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr"/>
       <c r="K41" s="3" t="inlineStr"/>
       <c r="L41" s="3" t="inlineStr">
         <is>
@@ -2384,7 +2380,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Meerab Fatima</t>
+          <t>Malahat Mardani</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2394,23 +2390,27 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Department of Computer Science, FAST National University of Computer and Emerging Sciences (FAST-NUCES)</t>
+          <t>Independent Researcher</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Recommender Systems; Natural Language Processing; Semantic Search and Information Retrieval; Large Language Models; Career and Skill-Gap Analysis</t>
-        </is>
-      </c>
-      <c r="F42" s="3" t="inlineStr"/>
+          <t>Machine Learning &amp; Deep Learning; Computer Vision; Medical Image Analysis; Biomedical Signal Processing (EEG); Model Reliability &amp; Generalization</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G42" s="3" t="inlineStr"/>
       <c r="H42" s="3" t="inlineStr"/>
-      <c r="I42" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J42" s="3" t="inlineStr"/>
+      <c r="I42" s="3" t="inlineStr"/>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K42" s="3" t="inlineStr"/>
       <c r="L42" s="3" t="inlineStr">
         <is>
@@ -2424,7 +2424,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Malahat Mardani</t>
+          <t>Mounes Mardani</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2468,7 +2468,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Mounes Mardani</t>
+          <t>Ramsha Khan</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2478,12 +2478,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Independent Researcher</t>
+          <t>University of Lahore</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning &amp; Deep Learning; Computer Vision; Medical Image Analysis; Biomedical Signal Processing (EEG); Model Reliability &amp; Generalization</t>
+          <t>AI for health; Biomedical research; Molecular medicine; Virology &amp; infectious diseases; AI in healthcare; Bioinformatics</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -2494,11 +2494,7 @@
       <c r="G44" s="3" t="inlineStr"/>
       <c r="H44" s="3" t="inlineStr"/>
       <c r="I44" s="3" t="inlineStr"/>
-      <c r="J44" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="J44" s="3" t="inlineStr"/>
       <c r="K44" s="3" t="inlineStr"/>
       <c r="L44" s="3" t="inlineStr">
         <is>
@@ -2512,7 +2508,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Ramsha Khan</t>
+          <t>Ali Hasnain</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2522,12 +2518,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>University of Lahore</t>
+          <t>Department of Software Engineering, University of Sahiwal</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>AI for health; Biomedical research; Molecular medicine; Virology &amp; infectious diseases; AI in healthcare; Bioinformatics</t>
+          <t>Computer vision; Medical AI; Large language models; Agentic AI; Deep learning</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
@@ -2535,10 +2531,18 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G45" s="3" t="inlineStr"/>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="H45" s="3" t="inlineStr"/>
       <c r="I45" s="3" t="inlineStr"/>
-      <c r="J45" s="3" t="inlineStr"/>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K45" s="3" t="inlineStr"/>
       <c r="L45" s="3" t="inlineStr">
         <is>
@@ -2552,7 +2556,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Ali Hasnain</t>
+          <t>Bilal Aslam</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2560,14 +2564,10 @@
           <t>Students &amp; Researchers</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>Department of Software Engineering, University of Sahiwal</t>
-        </is>
-      </c>
+      <c r="D46" t="inlineStr"/>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Computer vision; Medical AI; Large language models; Agentic AI; Deep learning</t>
+          <t>Machine learning; Deep learning; Healthcare AI; IoMT; Trustworthy AI</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
@@ -2575,11 +2575,7 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G46" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G46" s="3" t="inlineStr"/>
       <c r="H46" s="3" t="inlineStr"/>
       <c r="I46" s="3" t="inlineStr"/>
       <c r="J46" s="3" t="inlineStr">
@@ -2588,11 +2584,7 @@
         </is>
       </c>
       <c r="K46" s="3" t="inlineStr"/>
-      <c r="L46" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="L46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2600,7 +2592,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Bilal Aslam</t>
+          <t>Aittezaz Ahmad</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2611,14 +2603,10 @@
       <c r="D47" t="inlineStr"/>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Machine learning; Deep learning; Healthcare AI; IoMT; Trustworthy AI</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Reliability Engineering; Artificial Intelligence; Risk Assessment; Machine Learning–Assisted Optimization; Intelligent Monitoring</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr"/>
       <c r="G47" s="3" t="inlineStr"/>
       <c r="H47" s="3" t="inlineStr"/>
       <c r="I47" s="3" t="inlineStr"/>
@@ -2628,86 +2616,54 @@
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr"/>
-      <c r="L47" s="3" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Aittezaz Ahmad</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Students &amp; Researchers</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>Reliability Engineering; Artificial Intelligence; Risk Assessment; Machine Learning–Assisted Optimization; Intelligent Monitoring</t>
-        </is>
-      </c>
-      <c r="F48" s="3" t="inlineStr"/>
-      <c r="G48" s="3" t="inlineStr"/>
-      <c r="H48" s="3" t="inlineStr"/>
-      <c r="I48" s="3" t="inlineStr"/>
-      <c r="J48" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="K48" s="3" t="inlineStr"/>
-      <c r="L48" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
+      <c r="L47" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr"/>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Total (current)</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr"/>
+      <c r="D49" s="4" t="inlineStr"/>
+      <c r="E49" s="4" t="inlineStr"/>
+      <c r="F49" s="4">
+        <f>COUNTIF(F2:F47,"x")</f>
+        <v/>
+      </c>
+      <c r="G49" s="4">
+        <f>COUNTIF(G2:G47,"x")</f>
+        <v/>
+      </c>
+      <c r="H49" s="4">
+        <f>COUNTIF(H2:H47,"x")</f>
+        <v/>
+      </c>
+      <c r="I49" s="4">
+        <f>COUNTIF(I2:I47,"x")</f>
+        <v/>
+      </c>
+      <c r="J49" s="4">
+        <f>COUNTIF(J2:J47,"x")</f>
+        <v/>
+      </c>
+      <c r="K49" s="4">
+        <f>COUNTIF(K2:K47,"x")</f>
+        <v/>
+      </c>
+      <c r="L49" s="4">
+        <f>COUNTIF(L2:L47,"x")</f>
+        <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="inlineStr"/>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>Total (current)</t>
-        </is>
-      </c>
-      <c r="C50" s="4" t="inlineStr"/>
-      <c r="D50" s="4" t="inlineStr"/>
-      <c r="E50" s="4" t="inlineStr"/>
-      <c r="F50" s="4">
-        <f>COUNTIF(F2:F48,"x")</f>
-        <v/>
-      </c>
-      <c r="G50" s="4">
-        <f>COUNTIF(G2:G48,"x")</f>
-        <v/>
-      </c>
-      <c r="H50" s="4">
-        <f>COUNTIF(H2:H48,"x")</f>
-        <v/>
-      </c>
-      <c r="I50" s="4">
-        <f>COUNTIF(I2:I48,"x")</f>
-        <v/>
-      </c>
-      <c r="J50" s="4">
-        <f>COUNTIF(J2:J48,"x")</f>
-        <v/>
-      </c>
-      <c r="K50" s="4">
-        <f>COUNTIF(K2:K48,"x")</f>
-        <v/>
-      </c>
-      <c r="L50" s="4">
-        <f>COUNTIF(L2:L48,"x")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr"/>
-      <c r="B51" t="inlineStr">
+      <c r="A50" t="inlineStr"/>
+      <c r="B50" t="inlineStr">
         <is>
           <t>Mark "x" in each area a member belongs to</t>
         </is>

</xml_diff>

<commit_message>
Add Roya Haghighatjou to Students & Researchers
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SYNTERA-member-areas.xlsx
+++ b/SYNTERA-member-areas.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1592,7 +1592,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Javeria Iqbal</t>
+          <t>Roya Haghighatjou</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1602,33 +1602,29 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Department of Computer Science, National University of Computer and Emerging Sciences, Islamabad</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr"/>
+          <t>Independent Researcher</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Digital and psychological health interventions; Mental health; Aging, geriatric nursing and neurocognitive health; Cardiovascular nursing; Emergency and critical care nursing</t>
+        </is>
+      </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr"/>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="H24" s="3" t="inlineStr"/>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J24" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I24" s="3" t="inlineStr"/>
+      <c r="J24" s="3" t="inlineStr"/>
       <c r="K24" s="3" t="inlineStr"/>
-      <c r="L24" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="L24" s="3" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1636,7 +1632,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Damilare Ogunjobi</t>
+          <t>Javeria Iqbal</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1646,22 +1642,22 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Department of Data Science and Analytics, BI Norwegian Business School, Oslo</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Cybersecurity; Machine Learning; Networking &amp; IoT; Artificial Intelligence; Trustworthy AI</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr"/>
+          <t>Department of Computer Science, National University of Computer and Emerging Sciences, Islamabad</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G25" s="3" t="inlineStr"/>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="I25" s="3" t="inlineStr"/>
+      <c r="H25" s="3" t="inlineStr"/>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1680,7 +1676,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Nazmul Hossain</t>
+          <t>Damilare Ogunjobi</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1690,28 +1686,28 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Penston Academy of International Studies, Dhaka</t>
+          <t>Department of Data Science and Analytics, BI Norwegian Business School, Oslo</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Cybersecurity; Network Security; Data Privacy and Security; Wireless Networks and Communication Protocols; Human-AI Interactions</t>
+          <t>Cybersecurity; Machine Learning; Networking &amp; IoT; Artificial Intelligence; Trustworthy AI</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr"/>
       <c r="G26" s="3" t="inlineStr"/>
-      <c r="H26" s="3" t="inlineStr"/>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I26" s="3" t="inlineStr"/>
       <c r="J26" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="K26" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K26" s="3" t="inlineStr"/>
       <c r="L26" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1724,7 +1720,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Arooj Fatima</t>
+          <t>Nazmul Hossain</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1734,26 +1730,18 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Department of Computer Science, University of Wah, Wah Cantt; Govt. Graduate College for Women, Chakwal</t>
+          <t>Penston Academy of International Studies, Dhaka</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning; Deep Learning; Cybersecurity; Explainable AI (XAI); Trustworthy AI</t>
-        </is>
-      </c>
-      <c r="F27" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Cybersecurity; Network Security; Data Privacy and Security; Wireless Networks and Communication Protocols; Human-AI Interactions</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr"/>
       <c r="G27" s="3" t="inlineStr"/>
       <c r="H27" s="3" t="inlineStr"/>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I27" s="3" t="inlineStr"/>
       <c r="J27" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1776,7 +1764,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Tobias Romano</t>
+          <t>Arooj Fatima</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1786,12 +1774,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>UNICEN</t>
+          <t>Department of Computer Science, University of Wah, Wah Cantt; Govt. Graduate College for Women, Chakwal</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Agriculture; Computer Vision; Machine Learning; Robotics; Autonomous Systems</t>
+          <t>Machine Learning; Deep Learning; Cybersecurity; Explainable AI (XAI); Trustworthy AI</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -1800,18 +1788,22 @@
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr"/>
-      <c r="H28" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="I28" s="3" t="inlineStr"/>
+      <c r="H28" s="3" t="inlineStr"/>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="K28" s="3" t="inlineStr"/>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1824,7 +1816,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Shiva Jahanaray</t>
+          <t>Tobias Romano</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1834,12 +1826,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Independent Researcher</t>
+          <t>UNICEN</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Artificial Intelligence; Machine Learning; Deep Learning; Multimodal Learning; Biomedical AI</t>
+          <t>Agriculture; Computer Vision; Machine Learning; Robotics; Autonomous Systems</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -1848,7 +1840,11 @@
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr"/>
-      <c r="H29" s="3" t="inlineStr"/>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="I29" s="3" t="inlineStr"/>
       <c r="J29" s="3" t="inlineStr">
         <is>
@@ -1868,7 +1864,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Furqan Ahmad</t>
+          <t>Shiva Jahanaray</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1883,7 +1879,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>AIoT; Edge computing; TinyML; SDN &amp; network automation; Smart healthcare</t>
+          <t>Artificial Intelligence; Machine Learning; Deep Learning; Multimodal Learning; Biomedical AI</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -1899,11 +1895,7 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K30" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K30" s="3" t="inlineStr"/>
       <c r="L30" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1916,7 +1908,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Muhammad Irfan Aslam</t>
+          <t>Furqan Ahmad</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1926,12 +1918,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>University of Education, Lahore</t>
+          <t>Independent Researcher</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Natural Language Processing; Deep Learning; Artificial Intelligence; Image Processing; Machine Learning</t>
+          <t>AIoT; Edge computing; TinyML; SDN &amp; network automation; Smart healthcare</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -1942,8 +1934,16 @@
       <c r="G31" s="3" t="inlineStr"/>
       <c r="H31" s="3" t="inlineStr"/>
       <c r="I31" s="3" t="inlineStr"/>
-      <c r="J31" s="3" t="inlineStr"/>
-      <c r="K31" s="3" t="inlineStr"/>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Sepehr Amooeinejad</t>
+          <t>Muhammad Irfan Aslam</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1966,12 +1966,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>School of Information Systems, Queensland University of Technology, Brisbane, QLD</t>
+          <t>University of Education, Lahore</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning; Sports Injury Prediction; Bibliometrics; Digital Health; Sports Analytics</t>
+          <t>Natural Language Processing; Deep Learning; Artificial Intelligence; Image Processing; Machine Learning</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Ghalib Nadeem</t>
+          <t>Sepehr Amooeinejad</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2006,36 +2006,24 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Independent Researcher</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr"/>
+          <t>School of Information Systems, Queensland University of Technology, Brisbane, QLD</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Machine Learning; Sports Injury Prediction; Bibliometrics; Digital Health; Sports Analytics</t>
+        </is>
+      </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G33" s="3" t="inlineStr"/>
+      <c r="H33" s="3" t="inlineStr"/>
       <c r="I33" s="3" t="inlineStr"/>
-      <c r="J33" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="K33" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="J33" s="3" t="inlineStr"/>
+      <c r="K33" s="3" t="inlineStr"/>
       <c r="L33" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -2048,7 +2036,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Nida Ali</t>
+          <t>Ghalib Nadeem</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2058,24 +2046,36 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Department of Skill Development and Leadership, The University of Lahore, Lahore</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>Corpus Linguistics; English for Specific Purposes; Text Analysis; Computer-Assisted Language Learning; Applied Linguistics</t>
-        </is>
-      </c>
-      <c r="F34" s="3" t="inlineStr"/>
-      <c r="G34" s="3" t="inlineStr"/>
-      <c r="H34" s="3" t="inlineStr"/>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J34" s="3" t="inlineStr"/>
-      <c r="K34" s="3" t="inlineStr"/>
+          <t>Independent Researcher</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr"/>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Hina Mehboob</t>
+          <t>Nida Ali</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2098,23 +2098,23 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>National University of Sciences and Technology (NUST), Islamabad</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr"/>
-      <c r="F35" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Department of Skill Development and Leadership, The University of Lahore, Lahore</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Corpus Linguistics; English for Specific Purposes; Text Analysis; Computer-Assisted Language Learning; Applied Linguistics</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr"/>
       <c r="G35" s="3" t="inlineStr"/>
       <c r="H35" s="3" t="inlineStr"/>
-      <c r="I35" s="3" t="inlineStr"/>
-      <c r="J35" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr"/>
       <c r="K35" s="3" t="inlineStr"/>
       <c r="L35" s="3" t="inlineStr">
         <is>
@@ -2128,7 +2128,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Hasanga Uyanhewage</t>
+          <t>Hina Mehboob</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2138,15 +2138,15 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Tesco Mobile, Tesco UK</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>Software engineering; Human–AI interaction; AI governance; Privacy &amp; data protection; Trust &amp; decision-making</t>
-        </is>
-      </c>
-      <c r="F36" s="3" t="inlineStr"/>
+          <t>National University of Sciences and Technology (NUST), Islamabad</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G36" s="3" t="inlineStr"/>
       <c r="H36" s="3" t="inlineStr"/>
       <c r="I36" s="3" t="inlineStr"/>
@@ -2168,7 +2168,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Malak Emziane</t>
+          <t>Hasanga Uyanhewage</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2178,19 +2178,15 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>University of Tipaza</t>
+          <t>Tesco Mobile, Tesco UK</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Quantum cryptography; IoT; AI; Secure 5G/6G networks</t>
-        </is>
-      </c>
-      <c r="F37" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Software engineering; Human–AI interaction; AI governance; Privacy &amp; data protection; Trust &amp; decision-making</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr"/>
       <c r="G37" s="3" t="inlineStr"/>
       <c r="H37" s="3" t="inlineStr"/>
       <c r="I37" s="3" t="inlineStr"/>
@@ -2199,11 +2195,7 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K37" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="K37" s="3" t="inlineStr"/>
       <c r="L37" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -2216,7 +2208,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Mohamadali Rezaeimanesh</t>
+          <t>Malak Emziane</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2226,15 +2218,19 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>School of Information Systems, Queensland University of Technology (QUT), Brisbane, QLD</t>
+          <t>University of Tipaza</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning; Artificial Intelligence; Extended Reality (XR); Cloud Computing</t>
-        </is>
-      </c>
-      <c r="F38" s="3" t="inlineStr"/>
+          <t>Quantum cryptography; IoT; AI; Secure 5G/6G networks</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G38" s="3" t="inlineStr"/>
       <c r="H38" s="3" t="inlineStr"/>
       <c r="I38" s="3" t="inlineStr"/>
@@ -2243,7 +2239,11 @@
           <t>x</t>
         </is>
       </c>
-      <c r="K38" s="3" t="inlineStr"/>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="L38" s="3" t="inlineStr">
         <is>
           <t>x</t>
@@ -2256,7 +2256,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Amir H. Malekijoo</t>
+          <t>Mohamadali Rezaeimanesh</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2266,19 +2266,15 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Independent Researcher</t>
+          <t>School of Information Systems, Queensland University of Technology (QUT), Brisbane, QLD</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Artificial Intelligence; Reinforcement Learning; Human-Computer Interaction; Pattern Recognition; Decision Making Theory</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Machine Learning; Artificial Intelligence; Extended Reality (XR); Cloud Computing</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr"/>
       <c r="G39" s="3" t="inlineStr"/>
       <c r="H39" s="3" t="inlineStr"/>
       <c r="I39" s="3" t="inlineStr"/>
@@ -2300,7 +2296,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Thiwanka Kaushalya Nagasanga</t>
+          <t>Amir H. Malekijoo</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2310,15 +2306,19 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>CQUniversity Australia</t>
+          <t>Independent Researcher</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Explainable AI (XAI); Human-AI Decision-Making; AI Agents; Software Engineering; Project Management</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="inlineStr"/>
+          <t>Artificial Intelligence; Reinforcement Learning; Human-Computer Interaction; Pattern Recognition; Decision Making Theory</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G40" s="3" t="inlineStr"/>
       <c r="H40" s="3" t="inlineStr"/>
       <c r="I40" s="3" t="inlineStr"/>
@@ -2340,7 +2340,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Meerab Fatima</t>
+          <t>Thiwanka Kaushalya Nagasanga</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2350,23 +2350,23 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Department of Computer Science, FAST National University of Computer and Emerging Sciences (FAST-NUCES)</t>
+          <t>CQUniversity Australia</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Recommender Systems; Natural Language Processing; Semantic Search and Information Retrieval; Large Language Models; Career and Skill-Gap Analysis</t>
+          <t>Explainable AI (XAI); Human-AI Decision-Making; AI Agents; Software Engineering; Project Management</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr"/>
       <c r="G41" s="3" t="inlineStr"/>
       <c r="H41" s="3" t="inlineStr"/>
-      <c r="I41" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="J41" s="3" t="inlineStr"/>
+      <c r="I41" s="3" t="inlineStr"/>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K41" s="3" t="inlineStr"/>
       <c r="L41" s="3" t="inlineStr">
         <is>
@@ -2380,7 +2380,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Malahat Mardani</t>
+          <t>Meerab Fatima</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2390,27 +2390,23 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Independent Researcher</t>
+          <t>Department of Computer Science, FAST National University of Computer and Emerging Sciences (FAST-NUCES)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Machine Learning &amp; Deep Learning; Computer Vision; Medical Image Analysis; Biomedical Signal Processing (EEG); Model Reliability &amp; Generalization</t>
-        </is>
-      </c>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+          <t>Recommender Systems; Natural Language Processing; Semantic Search and Information Retrieval; Large Language Models; Career and Skill-Gap Analysis</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr"/>
       <c r="G42" s="3" t="inlineStr"/>
       <c r="H42" s="3" t="inlineStr"/>
-      <c r="I42" s="3" t="inlineStr"/>
-      <c r="J42" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr"/>
       <c r="K42" s="3" t="inlineStr"/>
       <c r="L42" s="3" t="inlineStr">
         <is>
@@ -2424,7 +2420,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Mounes Mardani</t>
+          <t>Malahat Mardani</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2468,7 +2464,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Ramsha Khan</t>
+          <t>Mounes Mardani</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2478,12 +2474,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>University of Lahore</t>
+          <t>Independent Researcher</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>AI for health; Biomedical research; Molecular medicine; Virology &amp; infectious diseases; AI in healthcare; Bioinformatics</t>
+          <t>Machine Learning &amp; Deep Learning; Computer Vision; Medical Image Analysis; Biomedical Signal Processing (EEG); Model Reliability &amp; Generalization</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -2494,7 +2490,11 @@
       <c r="G44" s="3" t="inlineStr"/>
       <c r="H44" s="3" t="inlineStr"/>
       <c r="I44" s="3" t="inlineStr"/>
-      <c r="J44" s="3" t="inlineStr"/>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="K44" s="3" t="inlineStr"/>
       <c r="L44" s="3" t="inlineStr">
         <is>
@@ -2508,7 +2508,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Ali Hasnain</t>
+          <t>Ramsha Khan</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2518,12 +2518,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Department of Software Engineering, University of Sahiwal</t>
+          <t>University of Lahore</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Computer vision; Medical AI; Large language models; Agentic AI; Deep learning</t>
+          <t>AI for health; Biomedical research; Molecular medicine; Virology &amp; infectious diseases; AI in healthcare; Bioinformatics</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
@@ -2531,18 +2531,10 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="G45" s="3" t="inlineStr"/>
       <c r="H45" s="3" t="inlineStr"/>
       <c r="I45" s="3" t="inlineStr"/>
-      <c r="J45" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
+      <c r="J45" s="3" t="inlineStr"/>
       <c r="K45" s="3" t="inlineStr"/>
       <c r="L45" s="3" t="inlineStr">
         <is>
@@ -2556,7 +2548,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Bilal Aslam</t>
+          <t>Ali Hasnain</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2564,10 +2556,14 @@
           <t>Students &amp; Researchers</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Department of Software Engineering, University of Sahiwal</t>
+        </is>
+      </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Machine learning; Deep learning; Healthcare AI; IoMT; Trustworthy AI</t>
+          <t>Computer vision; Medical AI; Large language models; Agentic AI; Deep learning</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
@@ -2575,7 +2571,11 @@
           <t>x</t>
         </is>
       </c>
-      <c r="G46" s="3" t="inlineStr"/>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="H46" s="3" t="inlineStr"/>
       <c r="I46" s="3" t="inlineStr"/>
       <c r="J46" s="3" t="inlineStr">
@@ -2584,7 +2584,11 @@
         </is>
       </c>
       <c r="K46" s="3" t="inlineStr"/>
-      <c r="L46" s="3" t="inlineStr"/>
+      <c r="L46" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2592,7 +2596,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Aittezaz Ahmad</t>
+          <t>Bilal Aslam</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2603,10 +2607,14 @@
       <c r="D47" t="inlineStr"/>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Reliability Engineering; Artificial Intelligence; Risk Assessment; Machine Learning–Assisted Optimization; Intelligent Monitoring</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="inlineStr"/>
+          <t>Machine learning; Deep learning; Healthcare AI; IoMT; Trustworthy AI</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
       <c r="G47" s="3" t="inlineStr"/>
       <c r="H47" s="3" t="inlineStr"/>
       <c r="I47" s="3" t="inlineStr"/>
@@ -2616,54 +2624,86 @@
         </is>
       </c>
       <c r="K47" s="3" t="inlineStr"/>
-      <c r="L47" s="3" t="inlineStr">
-        <is>
-          <t>x</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr"/>
-      <c r="B49" s="4" t="inlineStr">
+      <c r="L47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Aittezaz Ahmad</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Students &amp; Researchers</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>Reliability Engineering; Artificial Intelligence; Risk Assessment; Machine Learning–Assisted Optimization; Intelligent Monitoring</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr"/>
+      <c r="G48" s="3" t="inlineStr"/>
+      <c r="H48" s="3" t="inlineStr"/>
+      <c r="I48" s="3" t="inlineStr"/>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="K48" s="3" t="inlineStr"/>
+      <c r="L48" s="3" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr"/>
+      <c r="B50" s="4" t="inlineStr">
         <is>
           <t>Total (current)</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr"/>
-      <c r="D49" s="4" t="inlineStr"/>
-      <c r="E49" s="4" t="inlineStr"/>
-      <c r="F49" s="4">
-        <f>COUNTIF(F2:F47,"x")</f>
+      <c r="C50" s="4" t="inlineStr"/>
+      <c r="D50" s="4" t="inlineStr"/>
+      <c r="E50" s="4" t="inlineStr"/>
+      <c r="F50" s="4">
+        <f>COUNTIF(F2:F48,"x")</f>
         <v/>
       </c>
-      <c r="G49" s="4">
-        <f>COUNTIF(G2:G47,"x")</f>
+      <c r="G50" s="4">
+        <f>COUNTIF(G2:G48,"x")</f>
         <v/>
       </c>
-      <c r="H49" s="4">
-        <f>COUNTIF(H2:H47,"x")</f>
+      <c r="H50" s="4">
+        <f>COUNTIF(H2:H48,"x")</f>
         <v/>
       </c>
-      <c r="I49" s="4">
-        <f>COUNTIF(I2:I47,"x")</f>
+      <c r="I50" s="4">
+        <f>COUNTIF(I2:I48,"x")</f>
         <v/>
       </c>
-      <c r="J49" s="4">
-        <f>COUNTIF(J2:J47,"x")</f>
+      <c r="J50" s="4">
+        <f>COUNTIF(J2:J48,"x")</f>
         <v/>
       </c>
-      <c r="K49" s="4">
-        <f>COUNTIF(K2:K47,"x")</f>
+      <c r="K50" s="4">
+        <f>COUNTIF(K2:K48,"x")</f>
         <v/>
       </c>
-      <c r="L49" s="4">
-        <f>COUNTIF(L2:L47,"x")</f>
+      <c r="L50" s="4">
+        <f>COUNTIF(L2:L48,"x")</f>
         <v/>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" t="inlineStr"/>
-      <c r="B50" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr"/>
+      <c r="B51" t="inlineStr">
         <is>
           <t>Mark "x" in each area a member belongs to</t>
         </is>

</xml_diff>